<commit_message>
Sync 2026-07-02 08:37 - add tasks 181-232 (52 new KII tasks)
</commit_message>
<xml_diff>
--- a/project_time_sheet.xlsx
+++ b/project_time_sheet.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30131"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="2175" documentId="11_3E36CF56B8E44E068221A0921DFEBA9330CC02F1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7302FB0B-EFE3-4B09-BD3B-805310FDE20E}"/>
+  <xr:revisionPtr revIDLastSave="2607" documentId="11_3E36CF56B8E44E068221A0921DFEBA9330CC02F1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3EC30897-F0CD-4D6B-ADBA-7D9CF6C926C3}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="📋 Instructions" sheetId="3" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1046" uniqueCount="320">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1419" uniqueCount="456">
   <si>
     <t xml:space="preserve">  Project Time Sheet — User Guide</t>
   </si>
@@ -981,6 +981,414 @@
   </si>
   <si>
     <t>ashiqul-abi, dilinaabi</t>
+  </si>
+  <si>
+    <t>Start and Stop buttons not working</t>
+  </si>
+  <si>
+    <t>Start and Stop buttons do not respond when pressed on the home page</t>
+  </si>
+  <si>
+    <t>ui,bug</t>
+  </si>
+  <si>
+    <t>Run button does not start the system</t>
+  </si>
+  <si>
+    <t>When the run button is pressed, the system does not start</t>
+  </si>
+  <si>
+    <t>Alarm should display when safety is active and run is pressed</t>
+  </si>
+  <si>
+    <t>System should display an alarm when safety interlock is active and user attempts to run</t>
+  </si>
+  <si>
+    <t>ui,safety</t>
+  </si>
+  <si>
+    <t>Safety active but system appears running when run is pressed</t>
+  </si>
+  <si>
+    <t>When safety is active, pressing run should not allow the system to appear to be running</t>
+  </si>
+  <si>
+    <t>ui,safety,bug</t>
+  </si>
+  <si>
+    <t>Home page settings panel issues</t>
+  </si>
+  <si>
+    <t>Settings panel on home page needs review and fixes</t>
+  </si>
+  <si>
+    <t>ui</t>
+  </si>
+  <si>
+    <t>Tools tab showing in Conveyor tab - move to Advanced Settings</t>
+  </si>
+  <si>
+    <t>Tools UI component is incorrectly placed in the Conveyor tab; should be moved to Advanced Settings</t>
+  </si>
+  <si>
+    <t>ui,ux</t>
+  </si>
+  <si>
+    <t>Conveyor tab missing conveyor speed - DB record missing</t>
+  </si>
+  <si>
+    <t>Conveyor tab does not show conveyor speed; DB record for this setting appears to be missing</t>
+  </si>
+  <si>
+    <t>ui,bug,db</t>
+  </si>
+  <si>
+    <t>Emergency stop from Robot not displayed in KII UI status bar</t>
+  </si>
+  <si>
+    <t>No indication of emergency stops originating from the Robot is shown in the KII top status bar</t>
+  </si>
+  <si>
+    <t>Home screen UI should display robot status</t>
+  </si>
+  <si>
+    <t>Add robot status indicators to the home screen</t>
+  </si>
+  <si>
+    <t>Logs not updating on main page</t>
+  </si>
+  <si>
+    <t>The log view on the main/home page is not refreshing or updating in real time</t>
+  </si>
+  <si>
+    <t>Remove or hide language selector (internationalization)</t>
+  </si>
+  <si>
+    <t>Language selector should be hidden; internationalization not needed for current scope</t>
+  </si>
+  <si>
+    <t>Add production rates and scoring rates from KI</t>
+  </si>
+  <si>
+    <t>Bring production rates and scoring rates display from KI into the home page</t>
+  </si>
+  <si>
+    <t>ui,feature</t>
+  </si>
+  <si>
+    <t>Changeable conveyor speed from UI</t>
+  </si>
+  <si>
+    <t>Allow operator to change conveyor speed directly from the UI</t>
+  </si>
+  <si>
+    <t>Live badge should show offline when system not running</t>
+  </si>
+  <si>
+    <t>Replace or remove the live badge; show offline state when system is not running</t>
+  </si>
+  <si>
+    <t>Home screen preview rotation - portrait image</t>
+  </si>
+  <si>
+    <t>Home screen scan preview image should display in portrait orientation</t>
+  </si>
+  <si>
+    <t>Universal error popup for any errors - TBD</t>
+  </si>
+  <si>
+    <t>Implement a universal popup component to display any system errors consistently; design TBD</t>
+  </si>
+  <si>
+    <t>Recipe preview not showing cuts [bug]</t>
+  </si>
+  <si>
+    <t>Recipe preview is not working and does not display cut lines</t>
+  </si>
+  <si>
+    <t>ui,bug,recipes</t>
+  </si>
+  <si>
+    <t>Recipe edit - validate conveyor speed and fix page navigation</t>
+  </si>
+  <si>
+    <t>Validate conveyor speed field on recipe edit page; fix normal navigation flow to the page</t>
+  </si>
+  <si>
+    <t>Add text labels to recipe icons</t>
+  </si>
+  <si>
+    <t>Recipe icon buttons need visible text labels for clarity</t>
+  </si>
+  <si>
+    <t>ui,ux,recipes</t>
+  </si>
+  <si>
+    <t>Recipe wizard - bind client name and creation date on UI</t>
+  </si>
+  <si>
+    <t>Left side of recipe wizard should display bound client name and creation date</t>
+  </si>
+  <si>
+    <t>ui,recipes</t>
+  </si>
+  <si>
+    <t>Log search not working</t>
+  </si>
+  <si>
+    <t>Log search functionality is broken; logs should be searchable</t>
+  </si>
+  <si>
+    <t>ui,bug,logs</t>
+  </si>
+  <si>
+    <t>Maintenance - hide 2D camera sensor</t>
+  </si>
+  <si>
+    <t>Hide the 2D camera entry from the sensors section on the maintenance page</t>
+  </si>
+  <si>
+    <t>ashiqul-abi, dilinaabi, MauricioDuqueABI</t>
+  </si>
+  <si>
+    <t>ui,maintenance</t>
+  </si>
+  <si>
+    <t>Maintenance - bind 3D camera image and IP address</t>
+  </si>
+  <si>
+    <t>3D camera image and IP address should be data-bound and displayed correctly on maintenance page</t>
+  </si>
+  <si>
+    <t>Maintenance - show health status for Robot, 3D cameras, Ultrasonic, Pump, Conveyor</t>
+  </si>
+  <si>
+    <t>Display health indicators for all major components on the maintenance page including sequential conveyor running status</t>
+  </si>
+  <si>
+    <t>ui,maintenance,feature</t>
+  </si>
+  <si>
+    <t>Maintenance Robot - add installation date and last maintenance date inputs</t>
+  </si>
+  <si>
+    <t>Add input fields for installation date and last maintenance date; store robot offsets in DB</t>
+  </si>
+  <si>
+    <t>ui,maintenance,db</t>
+  </si>
+  <si>
+    <t>Maintenance Robot - hide working hours</t>
+  </si>
+  <si>
+    <t>Working hours field should be hidden on the robot maintenance page for now</t>
+  </si>
+  <si>
+    <t>Maintenance Robot - hide right side panel</t>
+  </si>
+  <si>
+    <t>Right side panel on the robot maintenance page should be hidden</t>
+  </si>
+  <si>
+    <t>Maintenance 3D cameras - hide page, implement camera blink ID, add calibration tool</t>
+  </si>
+  <si>
+    <t>3D cameras maintenance page: hide until XML config submitted; implement camera identification blink; add calibration tool</t>
+  </si>
+  <si>
+    <t>ui,maintenance,3d-camera</t>
+  </si>
+  <si>
+    <t>Maintenance 3D cameras - update camera image</t>
+  </si>
+  <si>
+    <t>Update/replace the camera image displayed on the 3D cameras maintenance page</t>
+  </si>
+  <si>
+    <t>Maintenance Pump - hide right side panel</t>
+  </si>
+  <si>
+    <t>Right side panel on the pump maintenance page should be hidden</t>
+  </si>
+  <si>
+    <t>Production Statistics - redesign pages</t>
+  </si>
+  <si>
+    <t>Production Statistics pages need a full redesign; design TBD</t>
+  </si>
+  <si>
+    <t>Last Images - pending test</t>
+  </si>
+  <si>
+    <t>Last Images feature is pending testing; check and verify later</t>
+  </si>
+  <si>
+    <t>testing</t>
+  </si>
+  <si>
+    <t>User management - fix threading issue causing page load error</t>
+  </si>
+  <si>
+    <t>User management page fails to load due to a threading issue; only loads successfully once</t>
+  </si>
+  <si>
+    <t>User Actions - hide superadmin and fix duplicate admin accounts</t>
+  </si>
+  <si>
+    <t>Hide the superadmin user from user selection; resolve duplicate admin and Admin entries</t>
+  </si>
+  <si>
+    <t>ui,bug,security</t>
+  </si>
+  <si>
+    <t>Engineering Settings - fix advanced settings tab height and button styles</t>
+  </si>
+  <si>
+    <t>Advanced settings tab should match page height; fix button design and styles</t>
+  </si>
+  <si>
+    <t>Engineering Settings - bind tools in tool settings page</t>
+  </si>
+  <si>
+    <t>Tool settings page should have all tools properly data-bound</t>
+  </si>
+  <si>
+    <t>Engineering Settings - fix layout and fonts</t>
+  </si>
+  <si>
+    <t>Fix page layout issues and font consistency in Engineering Settings</t>
+  </si>
+  <si>
+    <t>Engineering Settings - replace scrolling with page-by-page navigation</t>
+  </si>
+  <si>
+    <t>Remove vertical scrolling from settings; implement paginated navigation instead</t>
+  </si>
+  <si>
+    <t>Move Incident Reports to main navigation bar bottom</t>
+  </si>
+  <si>
+    <t>Incident reports section should be accessible from the bottom of the main navigation bar</t>
+  </si>
+  <si>
+    <t>Move Documentation to main navigation bar bottom</t>
+  </si>
+  <si>
+    <t>Documentation section should be accessible from the bottom of the main navigation bar</t>
+  </si>
+  <si>
+    <t>Find and update Incident and Documentation pages from GitHub</t>
+  </si>
+  <si>
+    <t>Locate Incident and Documentation page code in GitHub and bring to latest codebase</t>
+  </si>
+  <si>
+    <t>dev</t>
+  </si>
+  <si>
+    <t>Tools - add ability to create new tools and manage Tool IDs</t>
+  </si>
+  <si>
+    <t>No UI exists to create new tools or Tool IDs; implement tool creation with proper ID separation and management</t>
+  </si>
+  <si>
+    <t>feature,tools</t>
+  </si>
+  <si>
+    <t>Backend - update OPC server to EyeQ version for Katana</t>
+  </si>
+  <si>
+    <t>Bring OPC server for Katana up to the same version used in EyeQ</t>
+  </si>
+  <si>
+    <t>backend,opc</t>
+  </si>
+  <si>
+    <t>Backend - add toggle between robot controller and PLC for specific tags</t>
+  </si>
+  <si>
+    <t>Katana should support switching between robot controller and PLC for selected OPC tags</t>
+  </si>
+  <si>
+    <t>Backend - recipe save/load centralized to SSOT</t>
+  </si>
+  <si>
+    <t>Recipe save and load logic was inconsistent between WPF and Blazor; now centralized to single source of truth</t>
+  </si>
+  <si>
+    <t>backend,recipes</t>
+  </si>
+  <si>
+    <t>Completed 2026-06-04</t>
+  </si>
+  <si>
+    <t>Backend - permission hidden features set to readonly</t>
+  </si>
+  <si>
+    <t>Hidden features behind permissions are now set to readonly mode</t>
+  </si>
+  <si>
+    <t>backend,security</t>
+  </si>
+  <si>
+    <t>Robot - keep RAPID code at latest version</t>
+  </si>
+  <si>
+    <t>Ensure RAPID code is always maintained at the latest stable version</t>
+  </si>
+  <si>
+    <t>robot,rapid</t>
+  </si>
+  <si>
+    <t>Robot - error and stop when current tool is blank</t>
+  </si>
+  <si>
+    <t>If the current tool field is blank when Katana starts, it should raise an error and stop</t>
+  </si>
+  <si>
+    <t>robot,safety,bug</t>
+  </si>
+  <si>
+    <t>Robot - Katana start: robot stuck in semistatic RAPID</t>
+  </si>
+  <si>
+    <t>When Katana starts, the robot never starts and gets stuck in semistatic RAPID state</t>
+  </si>
+  <si>
+    <t>robot,bug</t>
+  </si>
+  <si>
+    <t>Discovered 2026-05-19</t>
+  </si>
+  <si>
+    <t>Robot - Cut Z-Depth=0 cuts product, height calculation error</t>
+  </si>
+  <si>
+    <t>Setting cut Z-Depth to 0 still cuts the product; likely a height calculation bug</t>
+  </si>
+  <si>
+    <t>Discovered 2026-06-02</t>
+  </si>
+  <si>
+    <t>PLC - OPC communication map and UDTs</t>
+  </si>
+  <si>
+    <t>Define and implement OPC communication map and UDT structures for Katana-PLC interface [in progress]</t>
+  </si>
+  <si>
+    <t>plc,opc</t>
+  </si>
+  <si>
+    <t>PLC - OPC multiple interfaces in Katana and PLC</t>
+  </si>
+  <si>
+    <t>Support multiple OPC interfaces between Katana application and PLC</t>
+  </si>
+  <si>
+    <t>Task unification</t>
+  </si>
+  <si>
+    <t>Unify all the tasks in one single file consolidation</t>
   </si>
 </sst>
 </file>
@@ -1332,7 +1740,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -1424,6 +1832,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
@@ -1634,6 +2043,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1990,22 +2403,22 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:3" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="32" t="s">
+      <c r="B2" s="33" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="32"/>
+      <c r="C2" s="33"/>
     </row>
     <row r="4" spans="2:3" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="33" t="s">
+      <c r="B4" s="34" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="33"/>
+      <c r="C4" s="34"/>
     </row>
     <row r="6" spans="2:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="31" t="s">
+      <c r="B6" s="32" t="s">
         <v>2</v>
       </c>
-      <c r="C6" s="31"/>
+      <c r="C6" s="32"/>
     </row>
     <row r="7" spans="2:3" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="1" t="s">
@@ -2032,10 +2445,10 @@
       </c>
     </row>
     <row r="11" spans="2:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="31" t="s">
+      <c r="B11" s="32" t="s">
         <v>9</v>
       </c>
-      <c r="C11" s="31"/>
+      <c r="C11" s="32"/>
     </row>
     <row r="12" spans="2:3" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12" s="1" t="s">
@@ -2134,10 +2547,10 @@
       </c>
     </row>
     <row r="25" spans="2:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B25" s="31" t="s">
+      <c r="B25" s="32" t="s">
         <v>34</v>
       </c>
-      <c r="C25" s="31"/>
+      <c r="C25" s="32"/>
     </row>
     <row r="26" spans="2:3" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B26" s="1" t="s">
@@ -2188,10 +2601,10 @@
       </c>
     </row>
     <row r="33" spans="2:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B33" s="31" t="s">
+      <c r="B33" s="32" t="s">
         <v>47</v>
       </c>
-      <c r="C33" s="31"/>
+      <c r="C33" s="32"/>
     </row>
     <row r="34" spans="2:3" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B34" s="1" t="s">
@@ -2252,7 +2665,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M181"/>
+  <dimension ref="A1:M234"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="7.77734375" customWidth="1"/>
@@ -7638,6 +8051,1405 @@
       <c r="L181" s="22"/>
       <c r="M181" s="26" t="s">
         <v>309</v>
+      </c>
+    </row>
+    <row r="182" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A182">
+        <v>181</v>
+      </c>
+      <c r="B182" s="3" t="s">
+        <v>320</v>
+      </c>
+      <c r="C182" s="3" t="s">
+        <v>321</v>
+      </c>
+      <c r="D182" t="s">
+        <v>319</v>
+      </c>
+      <c r="E182" t="s">
+        <v>59</v>
+      </c>
+      <c r="F182" t="s">
+        <v>312</v>
+      </c>
+      <c r="K182" t="s">
+        <v>322</v>
+      </c>
+      <c r="M182" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="183" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A183">
+        <v>182</v>
+      </c>
+      <c r="B183" s="3" t="s">
+        <v>323</v>
+      </c>
+      <c r="C183" s="3" t="s">
+        <v>324</v>
+      </c>
+      <c r="D183" t="s">
+        <v>319</v>
+      </c>
+      <c r="E183" t="s">
+        <v>59</v>
+      </c>
+      <c r="F183" t="s">
+        <v>312</v>
+      </c>
+      <c r="K183" t="s">
+        <v>322</v>
+      </c>
+      <c r="M183" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="184" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A184">
+        <v>183</v>
+      </c>
+      <c r="B184" s="3" t="s">
+        <v>325</v>
+      </c>
+      <c r="C184" s="3" t="s">
+        <v>326</v>
+      </c>
+      <c r="D184" t="s">
+        <v>319</v>
+      </c>
+      <c r="E184" t="s">
+        <v>59</v>
+      </c>
+      <c r="F184" t="s">
+        <v>312</v>
+      </c>
+      <c r="K184" t="s">
+        <v>327</v>
+      </c>
+      <c r="M184" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="185" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A185">
+        <v>184</v>
+      </c>
+      <c r="B185" s="3" t="s">
+        <v>328</v>
+      </c>
+      <c r="C185" s="3" t="s">
+        <v>329</v>
+      </c>
+      <c r="D185" t="s">
+        <v>319</v>
+      </c>
+      <c r="E185" t="s">
+        <v>59</v>
+      </c>
+      <c r="F185" t="s">
+        <v>312</v>
+      </c>
+      <c r="K185" t="s">
+        <v>330</v>
+      </c>
+      <c r="M185" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="186" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A186">
+        <v>185</v>
+      </c>
+      <c r="B186" s="3" t="s">
+        <v>331</v>
+      </c>
+      <c r="C186" s="3" t="s">
+        <v>332</v>
+      </c>
+      <c r="D186" t="s">
+        <v>319</v>
+      </c>
+      <c r="E186" t="s">
+        <v>59</v>
+      </c>
+      <c r="F186" t="s">
+        <v>312</v>
+      </c>
+      <c r="K186" t="s">
+        <v>333</v>
+      </c>
+      <c r="M186" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="187" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A187">
+        <v>186</v>
+      </c>
+      <c r="B187" s="3" t="s">
+        <v>334</v>
+      </c>
+      <c r="C187" s="3" t="s">
+        <v>335</v>
+      </c>
+      <c r="D187" t="s">
+        <v>319</v>
+      </c>
+      <c r="E187" t="s">
+        <v>59</v>
+      </c>
+      <c r="F187" t="s">
+        <v>312</v>
+      </c>
+      <c r="K187" t="s">
+        <v>336</v>
+      </c>
+      <c r="M187" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="188" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A188">
+        <v>187</v>
+      </c>
+      <c r="B188" s="3" t="s">
+        <v>337</v>
+      </c>
+      <c r="C188" s="3" t="s">
+        <v>338</v>
+      </c>
+      <c r="D188" t="s">
+        <v>319</v>
+      </c>
+      <c r="E188" t="s">
+        <v>59</v>
+      </c>
+      <c r="F188" t="s">
+        <v>312</v>
+      </c>
+      <c r="K188" t="s">
+        <v>339</v>
+      </c>
+      <c r="M188" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="189" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A189">
+        <v>188</v>
+      </c>
+      <c r="B189" s="3" t="s">
+        <v>340</v>
+      </c>
+      <c r="C189" s="3" t="s">
+        <v>341</v>
+      </c>
+      <c r="D189" t="s">
+        <v>319</v>
+      </c>
+      <c r="E189" t="s">
+        <v>59</v>
+      </c>
+      <c r="F189" t="s">
+        <v>312</v>
+      </c>
+      <c r="K189" t="s">
+        <v>327</v>
+      </c>
+      <c r="M189" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="190" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A190">
+        <v>189</v>
+      </c>
+      <c r="B190" s="3" t="s">
+        <v>342</v>
+      </c>
+      <c r="C190" s="3" t="s">
+        <v>343</v>
+      </c>
+      <c r="D190" t="s">
+        <v>319</v>
+      </c>
+      <c r="E190" t="s">
+        <v>59</v>
+      </c>
+      <c r="F190" t="s">
+        <v>312</v>
+      </c>
+      <c r="K190" t="s">
+        <v>336</v>
+      </c>
+      <c r="M190" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="191" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A191">
+        <v>190</v>
+      </c>
+      <c r="B191" s="3" t="s">
+        <v>344</v>
+      </c>
+      <c r="C191" s="3" t="s">
+        <v>345</v>
+      </c>
+      <c r="D191" t="s">
+        <v>319</v>
+      </c>
+      <c r="E191" t="s">
+        <v>59</v>
+      </c>
+      <c r="F191" t="s">
+        <v>312</v>
+      </c>
+      <c r="K191" t="s">
+        <v>322</v>
+      </c>
+      <c r="M191" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="192" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A192">
+        <v>191</v>
+      </c>
+      <c r="B192" s="3" t="s">
+        <v>346</v>
+      </c>
+      <c r="C192" s="3" t="s">
+        <v>347</v>
+      </c>
+      <c r="D192" t="s">
+        <v>319</v>
+      </c>
+      <c r="E192" t="s">
+        <v>59</v>
+      </c>
+      <c r="F192" t="s">
+        <v>312</v>
+      </c>
+      <c r="K192" t="s">
+        <v>333</v>
+      </c>
+      <c r="M192" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="193" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A193">
+        <v>192</v>
+      </c>
+      <c r="B193" s="3" t="s">
+        <v>348</v>
+      </c>
+      <c r="C193" s="3" t="s">
+        <v>349</v>
+      </c>
+      <c r="D193" t="s">
+        <v>319</v>
+      </c>
+      <c r="E193" t="s">
+        <v>59</v>
+      </c>
+      <c r="F193" t="s">
+        <v>312</v>
+      </c>
+      <c r="K193" t="s">
+        <v>350</v>
+      </c>
+      <c r="M193" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="194" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A194">
+        <v>193</v>
+      </c>
+      <c r="B194" s="3" t="s">
+        <v>351</v>
+      </c>
+      <c r="C194" s="3" t="s">
+        <v>352</v>
+      </c>
+      <c r="D194" t="s">
+        <v>319</v>
+      </c>
+      <c r="E194" t="s">
+        <v>59</v>
+      </c>
+      <c r="F194" t="s">
+        <v>312</v>
+      </c>
+      <c r="K194" t="s">
+        <v>350</v>
+      </c>
+      <c r="M194" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="195" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A195">
+        <v>194</v>
+      </c>
+      <c r="B195" s="3" t="s">
+        <v>353</v>
+      </c>
+      <c r="C195" s="3" t="s">
+        <v>354</v>
+      </c>
+      <c r="D195" t="s">
+        <v>319</v>
+      </c>
+      <c r="E195" t="s">
+        <v>59</v>
+      </c>
+      <c r="F195" t="s">
+        <v>312</v>
+      </c>
+      <c r="K195" t="s">
+        <v>336</v>
+      </c>
+      <c r="M195" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="196" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A196">
+        <v>195</v>
+      </c>
+      <c r="B196" s="3" t="s">
+        <v>355</v>
+      </c>
+      <c r="C196" s="3" t="s">
+        <v>356</v>
+      </c>
+      <c r="D196" t="s">
+        <v>319</v>
+      </c>
+      <c r="E196" t="s">
+        <v>59</v>
+      </c>
+      <c r="F196" t="s">
+        <v>312</v>
+      </c>
+      <c r="K196" t="s">
+        <v>322</v>
+      </c>
+      <c r="M196" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="197" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A197">
+        <v>196</v>
+      </c>
+      <c r="B197" s="3" t="s">
+        <v>357</v>
+      </c>
+      <c r="C197" s="3" t="s">
+        <v>358</v>
+      </c>
+      <c r="D197" t="s">
+        <v>319</v>
+      </c>
+      <c r="E197" t="s">
+        <v>59</v>
+      </c>
+      <c r="F197" t="s">
+        <v>312</v>
+      </c>
+      <c r="K197" t="s">
+        <v>350</v>
+      </c>
+      <c r="M197" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="198" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A198">
+        <v>197</v>
+      </c>
+      <c r="B198" s="3" t="s">
+        <v>359</v>
+      </c>
+      <c r="C198" s="3" t="s">
+        <v>360</v>
+      </c>
+      <c r="D198" t="s">
+        <v>60</v>
+      </c>
+      <c r="E198" t="s">
+        <v>59</v>
+      </c>
+      <c r="F198" t="s">
+        <v>313</v>
+      </c>
+      <c r="K198" t="s">
+        <v>361</v>
+      </c>
+      <c r="M198" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="199" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A199">
+        <v>198</v>
+      </c>
+      <c r="B199" s="3" t="s">
+        <v>362</v>
+      </c>
+      <c r="C199" s="3" t="s">
+        <v>363</v>
+      </c>
+      <c r="D199" t="s">
+        <v>60</v>
+      </c>
+      <c r="E199" t="s">
+        <v>59</v>
+      </c>
+      <c r="F199" t="s">
+        <v>313</v>
+      </c>
+      <c r="K199" t="s">
+        <v>361</v>
+      </c>
+      <c r="M199" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="200" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A200">
+        <v>199</v>
+      </c>
+      <c r="B200" s="3" t="s">
+        <v>364</v>
+      </c>
+      <c r="C200" s="3" t="s">
+        <v>365</v>
+      </c>
+      <c r="D200" t="s">
+        <v>60</v>
+      </c>
+      <c r="E200" t="s">
+        <v>59</v>
+      </c>
+      <c r="F200" t="s">
+        <v>313</v>
+      </c>
+      <c r="K200" t="s">
+        <v>366</v>
+      </c>
+      <c r="M200" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="201" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A201">
+        <v>200</v>
+      </c>
+      <c r="B201" s="3" t="s">
+        <v>367</v>
+      </c>
+      <c r="C201" s="3" t="s">
+        <v>368</v>
+      </c>
+      <c r="D201" t="s">
+        <v>60</v>
+      </c>
+      <c r="E201" t="s">
+        <v>59</v>
+      </c>
+      <c r="F201" t="s">
+        <v>313</v>
+      </c>
+      <c r="K201" t="s">
+        <v>369</v>
+      </c>
+      <c r="M201" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="202" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A202">
+        <v>201</v>
+      </c>
+      <c r="B202" s="3" t="s">
+        <v>370</v>
+      </c>
+      <c r="C202" s="3" t="s">
+        <v>371</v>
+      </c>
+      <c r="D202" t="s">
+        <v>60</v>
+      </c>
+      <c r="E202" t="s">
+        <v>59</v>
+      </c>
+      <c r="F202" t="s">
+        <v>314</v>
+      </c>
+      <c r="K202" t="s">
+        <v>372</v>
+      </c>
+      <c r="M202" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="203" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A203">
+        <v>202</v>
+      </c>
+      <c r="B203" s="3" t="s">
+        <v>373</v>
+      </c>
+      <c r="C203" s="3" t="s">
+        <v>374</v>
+      </c>
+      <c r="D203" t="s">
+        <v>375</v>
+      </c>
+      <c r="E203" t="s">
+        <v>59</v>
+      </c>
+      <c r="F203" t="s">
+        <v>313</v>
+      </c>
+      <c r="K203" t="s">
+        <v>376</v>
+      </c>
+      <c r="M203" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="204" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A204">
+        <v>203</v>
+      </c>
+      <c r="B204" s="3" t="s">
+        <v>377</v>
+      </c>
+      <c r="C204" s="3" t="s">
+        <v>378</v>
+      </c>
+      <c r="D204" t="s">
+        <v>375</v>
+      </c>
+      <c r="E204" t="s">
+        <v>59</v>
+      </c>
+      <c r="F204" t="s">
+        <v>313</v>
+      </c>
+      <c r="K204" t="s">
+        <v>376</v>
+      </c>
+      <c r="M204" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="205" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A205">
+        <v>204</v>
+      </c>
+      <c r="B205" s="3" t="s">
+        <v>379</v>
+      </c>
+      <c r="C205" s="3" t="s">
+        <v>380</v>
+      </c>
+      <c r="D205" t="s">
+        <v>375</v>
+      </c>
+      <c r="E205" t="s">
+        <v>59</v>
+      </c>
+      <c r="F205" t="s">
+        <v>313</v>
+      </c>
+      <c r="K205" t="s">
+        <v>381</v>
+      </c>
+      <c r="M205" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="206" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A206">
+        <v>205</v>
+      </c>
+      <c r="B206" s="3" t="s">
+        <v>382</v>
+      </c>
+      <c r="C206" s="3" t="s">
+        <v>383</v>
+      </c>
+      <c r="D206" t="s">
+        <v>60</v>
+      </c>
+      <c r="E206" t="s">
+        <v>59</v>
+      </c>
+      <c r="F206" t="s">
+        <v>314</v>
+      </c>
+      <c r="K206" t="s">
+        <v>384</v>
+      </c>
+      <c r="M206" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="207" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A207">
+        <v>206</v>
+      </c>
+      <c r="B207" s="3" t="s">
+        <v>385</v>
+      </c>
+      <c r="C207" s="3" t="s">
+        <v>386</v>
+      </c>
+      <c r="D207" t="s">
+        <v>60</v>
+      </c>
+      <c r="E207" t="s">
+        <v>59</v>
+      </c>
+      <c r="F207" t="s">
+        <v>314</v>
+      </c>
+      <c r="K207" t="s">
+        <v>376</v>
+      </c>
+      <c r="M207" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="208" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A208">
+        <v>207</v>
+      </c>
+      <c r="B208" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="C208" s="3" t="s">
+        <v>388</v>
+      </c>
+      <c r="D208" t="s">
+        <v>60</v>
+      </c>
+      <c r="E208" t="s">
+        <v>59</v>
+      </c>
+      <c r="F208" t="s">
+        <v>314</v>
+      </c>
+      <c r="K208" t="s">
+        <v>376</v>
+      </c>
+      <c r="M208" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="209" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A209">
+        <v>208</v>
+      </c>
+      <c r="B209" s="3" t="s">
+        <v>389</v>
+      </c>
+      <c r="C209" s="3" t="s">
+        <v>390</v>
+      </c>
+      <c r="D209" t="s">
+        <v>61</v>
+      </c>
+      <c r="E209" t="s">
+        <v>59</v>
+      </c>
+      <c r="F209" t="s">
+        <v>313</v>
+      </c>
+      <c r="K209" t="s">
+        <v>391</v>
+      </c>
+      <c r="M209" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="210" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A210">
+        <v>209</v>
+      </c>
+      <c r="B210" s="3" t="s">
+        <v>392</v>
+      </c>
+      <c r="C210" s="3" t="s">
+        <v>393</v>
+      </c>
+      <c r="D210" t="s">
+        <v>61</v>
+      </c>
+      <c r="E210" t="s">
+        <v>59</v>
+      </c>
+      <c r="F210" t="s">
+        <v>313</v>
+      </c>
+      <c r="K210" t="s">
+        <v>391</v>
+      </c>
+      <c r="M210" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="211" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A211">
+        <v>210</v>
+      </c>
+      <c r="B211" s="3" t="s">
+        <v>394</v>
+      </c>
+      <c r="C211" s="3" t="s">
+        <v>395</v>
+      </c>
+      <c r="D211" t="s">
+        <v>58</v>
+      </c>
+      <c r="E211" t="s">
+        <v>59</v>
+      </c>
+      <c r="F211" t="s">
+        <v>314</v>
+      </c>
+      <c r="K211" t="s">
+        <v>376</v>
+      </c>
+      <c r="M211" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="212" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A212">
+        <v>211</v>
+      </c>
+      <c r="B212" s="3" t="s">
+        <v>396</v>
+      </c>
+      <c r="C212" s="3" t="s">
+        <v>397</v>
+      </c>
+      <c r="D212" t="s">
+        <v>58</v>
+      </c>
+      <c r="E212" t="s">
+        <v>59</v>
+      </c>
+      <c r="F212" t="s">
+        <v>314</v>
+      </c>
+      <c r="K212" t="s">
+        <v>350</v>
+      </c>
+      <c r="M212" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="213" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A213">
+        <v>212</v>
+      </c>
+      <c r="B213" s="3" t="s">
+        <v>398</v>
+      </c>
+      <c r="C213" s="3" t="s">
+        <v>399</v>
+      </c>
+      <c r="E213" t="s">
+        <v>59</v>
+      </c>
+      <c r="F213" t="s">
+        <v>314</v>
+      </c>
+      <c r="K213" t="s">
+        <v>400</v>
+      </c>
+      <c r="M213" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="214" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A214">
+        <v>213</v>
+      </c>
+      <c r="B214" s="3" t="s">
+        <v>401</v>
+      </c>
+      <c r="C214" s="3" t="s">
+        <v>402</v>
+      </c>
+      <c r="D214" t="s">
+        <v>61</v>
+      </c>
+      <c r="E214" t="s">
+        <v>59</v>
+      </c>
+      <c r="F214" t="s">
+        <v>314</v>
+      </c>
+      <c r="K214" t="s">
+        <v>322</v>
+      </c>
+      <c r="M214" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="215" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A215">
+        <v>214</v>
+      </c>
+      <c r="B215" s="3" t="s">
+        <v>403</v>
+      </c>
+      <c r="C215" s="3" t="s">
+        <v>404</v>
+      </c>
+      <c r="D215" t="s">
+        <v>60</v>
+      </c>
+      <c r="E215" t="s">
+        <v>59</v>
+      </c>
+      <c r="F215" t="s">
+        <v>314</v>
+      </c>
+      <c r="K215" t="s">
+        <v>405</v>
+      </c>
+      <c r="M215" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="216" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A216">
+        <v>215</v>
+      </c>
+      <c r="B216" s="3" t="s">
+        <v>406</v>
+      </c>
+      <c r="C216" s="3" t="s">
+        <v>407</v>
+      </c>
+      <c r="D216" t="s">
+        <v>60</v>
+      </c>
+      <c r="E216" t="s">
+        <v>59</v>
+      </c>
+      <c r="F216" t="s">
+        <v>312</v>
+      </c>
+      <c r="K216" t="s">
+        <v>336</v>
+      </c>
+      <c r="M216" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="217" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A217">
+        <v>216</v>
+      </c>
+      <c r="B217" s="3" t="s">
+        <v>408</v>
+      </c>
+      <c r="C217" s="3" t="s">
+        <v>409</v>
+      </c>
+      <c r="D217" t="s">
+        <v>60</v>
+      </c>
+      <c r="E217" t="s">
+        <v>59</v>
+      </c>
+      <c r="F217" t="s">
+        <v>312</v>
+      </c>
+      <c r="K217" t="s">
+        <v>350</v>
+      </c>
+      <c r="M217" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="218" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A218">
+        <v>217</v>
+      </c>
+      <c r="B218" s="3" t="s">
+        <v>410</v>
+      </c>
+      <c r="C218" s="3" t="s">
+        <v>411</v>
+      </c>
+      <c r="D218" t="s">
+        <v>60</v>
+      </c>
+      <c r="E218" t="s">
+        <v>59</v>
+      </c>
+      <c r="F218" t="s">
+        <v>312</v>
+      </c>
+      <c r="K218" t="s">
+        <v>336</v>
+      </c>
+      <c r="M218" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="219" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A219">
+        <v>218</v>
+      </c>
+      <c r="B219" s="3" t="s">
+        <v>412</v>
+      </c>
+      <c r="C219" s="3" t="s">
+        <v>413</v>
+      </c>
+      <c r="D219" t="s">
+        <v>60</v>
+      </c>
+      <c r="E219" t="s">
+        <v>59</v>
+      </c>
+      <c r="F219" t="s">
+        <v>312</v>
+      </c>
+      <c r="K219" t="s">
+        <v>336</v>
+      </c>
+      <c r="M219" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="220" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A220">
+        <v>219</v>
+      </c>
+      <c r="B220" s="3" t="s">
+        <v>414</v>
+      </c>
+      <c r="C220" s="3" t="s">
+        <v>415</v>
+      </c>
+      <c r="D220" t="s">
+        <v>60</v>
+      </c>
+      <c r="E220" t="s">
+        <v>59</v>
+      </c>
+      <c r="F220" t="s">
+        <v>314</v>
+      </c>
+      <c r="K220" t="s">
+        <v>336</v>
+      </c>
+      <c r="M220" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="221" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A221">
+        <v>220</v>
+      </c>
+      <c r="B221" s="3" t="s">
+        <v>416</v>
+      </c>
+      <c r="C221" s="3" t="s">
+        <v>417</v>
+      </c>
+      <c r="D221" t="s">
+        <v>60</v>
+      </c>
+      <c r="E221" t="s">
+        <v>59</v>
+      </c>
+      <c r="F221" t="s">
+        <v>314</v>
+      </c>
+      <c r="K221" t="s">
+        <v>336</v>
+      </c>
+      <c r="M221" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="222" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A222">
+        <v>221</v>
+      </c>
+      <c r="B222" s="3" t="s">
+        <v>418</v>
+      </c>
+      <c r="C222" s="3" t="s">
+        <v>419</v>
+      </c>
+      <c r="D222" t="s">
+        <v>60</v>
+      </c>
+      <c r="E222" t="s">
+        <v>59</v>
+      </c>
+      <c r="F222" t="s">
+        <v>314</v>
+      </c>
+      <c r="K222" t="s">
+        <v>420</v>
+      </c>
+      <c r="M222" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="223" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A223">
+        <v>222</v>
+      </c>
+      <c r="B223" s="3" t="s">
+        <v>421</v>
+      </c>
+      <c r="C223" s="3" t="s">
+        <v>422</v>
+      </c>
+      <c r="E223" t="s">
+        <v>59</v>
+      </c>
+      <c r="F223" t="s">
+        <v>312</v>
+      </c>
+      <c r="K223" t="s">
+        <v>423</v>
+      </c>
+      <c r="M223" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="224" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A224">
+        <v>223</v>
+      </c>
+      <c r="B224" s="3" t="s">
+        <v>424</v>
+      </c>
+      <c r="C224" s="3" t="s">
+        <v>425</v>
+      </c>
+      <c r="D224" t="s">
+        <v>61</v>
+      </c>
+      <c r="E224" t="s">
+        <v>59</v>
+      </c>
+      <c r="F224" t="s">
+        <v>312</v>
+      </c>
+      <c r="K224" t="s">
+        <v>426</v>
+      </c>
+      <c r="M224" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="225" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A225">
+        <v>224</v>
+      </c>
+      <c r="B225" s="3" t="s">
+        <v>427</v>
+      </c>
+      <c r="C225" s="3" t="s">
+        <v>428</v>
+      </c>
+      <c r="D225" t="s">
+        <v>61</v>
+      </c>
+      <c r="E225" t="s">
+        <v>59</v>
+      </c>
+      <c r="F225" t="s">
+        <v>312</v>
+      </c>
+      <c r="K225" t="s">
+        <v>426</v>
+      </c>
+      <c r="M225" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="226" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A226">
+        <v>225</v>
+      </c>
+      <c r="B226" s="3" t="s">
+        <v>429</v>
+      </c>
+      <c r="C226" s="3" t="s">
+        <v>430</v>
+      </c>
+      <c r="D226" t="s">
+        <v>61</v>
+      </c>
+      <c r="E226" t="s">
+        <v>73</v>
+      </c>
+      <c r="F226" t="s">
+        <v>313</v>
+      </c>
+      <c r="H226" s="31">
+        <v>46177</v>
+      </c>
+      <c r="K226" t="s">
+        <v>431</v>
+      </c>
+      <c r="L226" t="s">
+        <v>432</v>
+      </c>
+      <c r="M226" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="227" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A227">
+        <v>226</v>
+      </c>
+      <c r="B227" s="3" t="s">
+        <v>433</v>
+      </c>
+      <c r="C227" s="3" t="s">
+        <v>434</v>
+      </c>
+      <c r="D227" t="s">
+        <v>61</v>
+      </c>
+      <c r="E227" t="s">
+        <v>73</v>
+      </c>
+      <c r="F227" t="s">
+        <v>313</v>
+      </c>
+      <c r="H227" s="31">
+        <v>46177</v>
+      </c>
+      <c r="K227" t="s">
+        <v>435</v>
+      </c>
+      <c r="L227" t="s">
+        <v>432</v>
+      </c>
+      <c r="M227" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="228" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A228">
+        <v>227</v>
+      </c>
+      <c r="B228" s="3" t="s">
+        <v>436</v>
+      </c>
+      <c r="C228" s="3" t="s">
+        <v>437</v>
+      </c>
+      <c r="D228" t="s">
+        <v>58</v>
+      </c>
+      <c r="E228" t="s">
+        <v>59</v>
+      </c>
+      <c r="F228" t="s">
+        <v>312</v>
+      </c>
+      <c r="K228" t="s">
+        <v>438</v>
+      </c>
+      <c r="M228" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="229" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A229">
+        <v>228</v>
+      </c>
+      <c r="B229" s="3" t="s">
+        <v>439</v>
+      </c>
+      <c r="C229" s="3" t="s">
+        <v>440</v>
+      </c>
+      <c r="D229" t="s">
+        <v>58</v>
+      </c>
+      <c r="E229" t="s">
+        <v>59</v>
+      </c>
+      <c r="F229" t="s">
+        <v>312</v>
+      </c>
+      <c r="K229" t="s">
+        <v>441</v>
+      </c>
+      <c r="M229" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="230" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A230">
+        <v>229</v>
+      </c>
+      <c r="B230" s="3" t="s">
+        <v>442</v>
+      </c>
+      <c r="C230" s="3" t="s">
+        <v>443</v>
+      </c>
+      <c r="D230" t="s">
+        <v>58</v>
+      </c>
+      <c r="E230" t="s">
+        <v>59</v>
+      </c>
+      <c r="F230" t="s">
+        <v>312</v>
+      </c>
+      <c r="H230" s="31">
+        <v>46161</v>
+      </c>
+      <c r="K230" t="s">
+        <v>444</v>
+      </c>
+      <c r="L230" t="s">
+        <v>445</v>
+      </c>
+      <c r="M230" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="231" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A231">
+        <v>230</v>
+      </c>
+      <c r="B231" s="3" t="s">
+        <v>446</v>
+      </c>
+      <c r="C231" s="3" t="s">
+        <v>447</v>
+      </c>
+      <c r="D231" t="s">
+        <v>58</v>
+      </c>
+      <c r="E231" t="s">
+        <v>59</v>
+      </c>
+      <c r="F231" t="s">
+        <v>312</v>
+      </c>
+      <c r="H231" s="31">
+        <v>46175</v>
+      </c>
+      <c r="K231" t="s">
+        <v>444</v>
+      </c>
+      <c r="L231" t="s">
+        <v>448</v>
+      </c>
+      <c r="M231" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="232" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A232">
+        <v>231</v>
+      </c>
+      <c r="B232" s="3" t="s">
+        <v>449</v>
+      </c>
+      <c r="C232" s="3" t="s">
+        <v>450</v>
+      </c>
+      <c r="D232" t="s">
+        <v>58</v>
+      </c>
+      <c r="E232" t="s">
+        <v>62</v>
+      </c>
+      <c r="F232" t="s">
+        <v>312</v>
+      </c>
+      <c r="K232" t="s">
+        <v>451</v>
+      </c>
+      <c r="L232" t="s">
+        <v>62</v>
+      </c>
+      <c r="M232" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="233" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A233">
+        <v>232</v>
+      </c>
+      <c r="B233" s="3" t="s">
+        <v>452</v>
+      </c>
+      <c r="C233" s="3" t="s">
+        <v>453</v>
+      </c>
+      <c r="D233" t="s">
+        <v>58</v>
+      </c>
+      <c r="E233" t="s">
+        <v>59</v>
+      </c>
+      <c r="F233" t="s">
+        <v>312</v>
+      </c>
+      <c r="K233" t="s">
+        <v>451</v>
+      </c>
+      <c r="M233" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="234" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A234">
+        <v>233</v>
+      </c>
+      <c r="B234" s="3" t="s">
+        <v>454</v>
+      </c>
+      <c r="C234" s="3" t="s">
+        <v>455</v>
+      </c>
+      <c r="D234" t="s">
+        <v>58</v>
+      </c>
+      <c r="E234" t="s">
+        <v>62</v>
+      </c>
+      <c r="F234" t="s">
+        <v>312</v>
+      </c>
+      <c r="H234" s="31">
+        <v>46205</v>
+      </c>
+      <c r="M234" t="s">
+        <v>308</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Sync 2026-08-12: 3 new items (#418-420, GH #974-976), 398 Monday.com items updated
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/project_time_sheet.xlsx
+++ b/project_time_sheet.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30228"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="54122" documentId="11_3E36CF56B8E44E068221A0921DFEBA9330CC02F1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{97FABF22-ACA5-4D48-BD63-4959357EF8E2}"/>
+  <xr:revisionPtr revIDLastSave="56887" documentId="11_3E36CF56B8E44E068221A0921DFEBA9330CC02F1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E451D5F5-FE4A-4B21-8444-2A328EF660D0}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2213" uniqueCount="801">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2225" uniqueCount="804">
   <si>
     <t xml:space="preserve">  Project Time Sheet — User Guide</t>
   </si>
@@ -2440,6 +2440,15 @@
   </si>
   <si>
     <t>Documentation</t>
+  </si>
+  <si>
+    <t>Add labeling tool - EyeQ</t>
+  </si>
+  <si>
+    <t>Add steps for detection - EyeQ</t>
+  </si>
+  <si>
+    <t>Auto-trigger calibration -EyeQ</t>
   </si>
 </sst>
 </file>
@@ -15796,14 +15805,59 @@
       </c>
     </row>
     <row r="419" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A419">
+        <v>418</v>
+      </c>
+      <c r="B419" s="3" t="s">
+        <v>801</v>
+      </c>
+      <c r="D419" t="s">
+        <v>66</v>
+      </c>
+      <c r="E419" t="s">
+        <v>71</v>
+      </c>
+      <c r="F419" t="s">
+        <v>431</v>
+      </c>
       <c r="I419" s="42"/>
       <c r="J419" s="42"/>
     </row>
     <row r="420" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A420">
+        <v>419</v>
+      </c>
+      <c r="B420" s="3" t="s">
+        <v>802</v>
+      </c>
+      <c r="D420" t="s">
+        <v>66</v>
+      </c>
+      <c r="E420" t="s">
+        <v>71</v>
+      </c>
+      <c r="F420" t="s">
+        <v>431</v>
+      </c>
       <c r="I420" s="42"/>
       <c r="J420" s="42"/>
     </row>
     <row r="421" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A421">
+        <v>420</v>
+      </c>
+      <c r="B421" s="3" t="s">
+        <v>803</v>
+      </c>
+      <c r="D421" t="s">
+        <v>66</v>
+      </c>
+      <c r="E421" t="s">
+        <v>71</v>
+      </c>
+      <c r="F421" t="s">
+        <v>431</v>
+      </c>
       <c r="I421" s="42"/>
       <c r="J421" s="42"/>
     </row>
@@ -18237,26 +18291,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="2e20d828-e3fd-41fd-921c-fbe0ff523ae8">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="adfc7943-f9ee-4478-a01e-ebfcb6e54f53" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100959716F11FB6F9409089B98D1C11D330" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="bc55ac45923017d94ee4534da3224188">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="2e20d828-e3fd-41fd-921c-fbe0ff523ae8" xmlns:ns3="adfc7943-f9ee-4478-a01e-ebfcb6e54f53" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="5bc17ad4f23ab8382a0bb5b03decca58" ns2:_="" ns3:_="">
     <xsd:import namespace="2e20d828-e3fd-41fd-921c-fbe0ff523ae8"/>
@@ -18511,10 +18545,41 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="2e20d828-e3fd-41fd-921c-fbe0ff523ae8">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="adfc7943-f9ee-4478-a01e-ebfcb6e54f53" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{737DCCA1-99B2-40A5-A4E9-9FBBAC380C60}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5CE6A3B7-F954-4629-B802-2205DECE6851}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="2e20d828-e3fd-41fd-921c-fbe0ff523ae8"/>
+    <ds:schemaRef ds:uri="adfc7943-f9ee-4478-a01e-ebfcb6e54f53"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -18531,20 +18596,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5CE6A3B7-F954-4629-B802-2205DECE6851}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{737DCCA1-99B2-40A5-A4E9-9FBBAC380C60}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="2e20d828-e3fd-41fd-921c-fbe0ff523ae8"/>
-    <ds:schemaRef ds:uri="adfc7943-f9ee-4478-a01e-ebfcb6e54f53"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Add 8 Eye-Q V3 tasks (#467-#474): cleanup, metrology, and docs
GitHub issues ABI.Unity #1016-#1023, all Done/MauricioDuqueABI.
Monday.com subitems created under Eye-Q parent (11002499253).

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/project_time_sheet.xlsx
+++ b/project_time_sheet.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30228"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="65138" documentId="11_3E36CF56B8E44E068221A0921DFEBA9330CC02F1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BFD72DD4-FEAB-440C-85E4-CBD11C194469}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{169DDE66-1599-4C9B-93B3-BE14E466E66C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2460" uniqueCount="881">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2524" uniqueCount="913">
   <si>
     <t xml:space="preserve">  Project Time Sheet — User Guide</t>
   </si>
@@ -2680,6 +2680,102 @@
   </si>
   <si>
     <t>Phantom images in Engineering Settings should not be saveable; the save action should be blocked or disabled for phantom images.</t>
+  </si>
+  <si>
+    <t>Remove the standalone Detection page</t>
+  </si>
+  <si>
+    <t>Retire the dedicated /#detection screen; the classical product detector is reached as a Classical Product Detector node in the Workflow editor, fed by camera, upload, network source, crop or stitcher nodes.</t>
+  </si>
+  <si>
+    <t>cleanup,frontend,docs</t>
+  </si>
+  <si>
+    <t>Commit b2cf7ce (08:35). Touched ProductDetection.md, Workflow.md, README.md, index.html, docs/content.html. Net -46 lines.</t>
+  </si>
+  <si>
+    <t>Remove the Colour analysis view</t>
+  </si>
+  <si>
+    <t>Delete the Colour analysis screen, its rail entry, chart icon, export/clear controls and supporting JavaScript, plus 54 lines of now-unused CSS.</t>
+  </si>
+  <si>
+    <t>cleanup,frontend</t>
+  </si>
+  <si>
+    <t>Commit 37ca892 (12:41). index.html -86 lines, app.css -54. The /color-data and /export_color_csv endpoints were not removed.</t>
+  </si>
+  <si>
+    <t>API.md described views that no longer exist</t>
+  </si>
+  <si>
+    <t>Correct the GET / section: the page is documented as live stream, training, workflow, camera settings, settings, logs, system and documentation views, replacing the stale list of five.</t>
+  </si>
+  <si>
+    <t>docs</t>
+  </si>
+  <si>
+    <t>Commit 37ca892 (12:41). Documentation drift caught during the same cleanup.</t>
+  </si>
+  <si>
+    <t>No physical measurement from a stitched 2D image</t>
+  </si>
+  <si>
+    <t>Add a Planar World Metrology postprocess node: a four-point image-to-conveyor-plane homography that maps product contours into plane coordinates and outputs length_mm, width_mm, area_mm2 and a world-coordinate oriented box.</t>
+  </si>
+  <si>
+    <t>feature,workflow,metrology</t>
+  </si>
+  <si>
+    <t>Commit 78d2f08 (17:01). New planar_metrology in postprocess_nodes.py (+81).</t>
+  </si>
+  <si>
+    <t>No way to mark the calibrated reference plane</t>
+  </si>
+  <si>
+    <t>Extend the workflow ROI picker so the metrology node offers Select reference plane: mark the four corners of a known rectangular conveyor area and enter its physical width and height.</t>
+  </si>
+  <si>
+    <t>feature,frontend,workflow</t>
+  </si>
+  <si>
+    <t>Commit 78d2f08 (17:01), workflow.js (+38/-?). Reuses the existing crop ROI selector.</t>
+  </si>
+  <si>
+    <t>RealSense 3D Metrology accepted sources it cannot measure</t>
+  </si>
+  <si>
+    <t>Require an explicit RealSense depth source; reject Basler, RGB-only, uploaded and combined sources. Depth intrinsics come from the active RealSense runtime or can be entered manually.</t>
+  </si>
+  <si>
+    <t>bugfix,workflow,validation</t>
+  </si>
+  <si>
+    <t>Commit 78d2f08 (17:01), inference_nodes.py (+24).</t>
+  </si>
+  <si>
+    <t>Export node could not choose where output lands</t>
+  </si>
+  <si>
+    <t>Give the Export node an Output directory that accepts a typed path or the Image Archive Browse dialog, including drive navigation and New folder.</t>
+  </si>
+  <si>
+    <t>feature,workflow,frontend</t>
+  </si>
+  <si>
+    <t>Commit 78d2f08 (17:01), result_nodes.py and workflow.js.</t>
+  </si>
+  <si>
+    <t>New metrology and export behaviour undocumented</t>
+  </si>
+  <si>
+    <t>Document Planar World Metrology, the RealSense 3D Metrology source rules and the Export output directory in Workflow.md and the in-app documentation view.</t>
+  </si>
+  <si>
+    <t>docs,workflow</t>
+  </si>
+  <si>
+    <t>Commit 78d2f08 (17:01). Workflow.md (+20) and ui/docs/content.html (+3).</t>
   </si>
 </sst>
 </file>
@@ -3940,10 +4036,6 @@
 </namedSheetViews>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -4565,7 +4657,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:N997"/>
+  <dimension ref="A1:N1005"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="7.6640625" customWidth="1"/>
@@ -18226,25 +18318,305 @@
       <c r="I992" s="42"/>
       <c r="J992" s="42"/>
     </row>
-    <row r="993" spans="9:10" x14ac:dyDescent="0.3">
+    <row r="993" spans="1:13" x14ac:dyDescent="0.3">
       <c r="I993" s="42"/>
       <c r="J993" s="42"/>
     </row>
-    <row r="994" spans="9:10" x14ac:dyDescent="0.3">
+    <row r="994" spans="1:13" x14ac:dyDescent="0.3">
       <c r="I994" s="42"/>
       <c r="J994" s="42"/>
     </row>
-    <row r="995" spans="9:10" x14ac:dyDescent="0.3">
+    <row r="995" spans="1:13" x14ac:dyDescent="0.3">
       <c r="I995" s="42"/>
       <c r="J995" s="42"/>
     </row>
-    <row r="996" spans="9:10" x14ac:dyDescent="0.3">
+    <row r="996" spans="1:13" x14ac:dyDescent="0.3">
       <c r="I996" s="42"/>
       <c r="J996" s="42"/>
     </row>
-    <row r="997" spans="9:10" x14ac:dyDescent="0.3">
+    <row r="997" spans="1:13" x14ac:dyDescent="0.3">
       <c r="I997" s="42"/>
       <c r="J997" s="42"/>
+    </row>
+    <row r="998" spans="1:13" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A998">
+        <v>467</v>
+      </c>
+      <c r="B998" s="3" t="s">
+        <v>881</v>
+      </c>
+      <c r="C998" s="3" t="s">
+        <v>882</v>
+      </c>
+      <c r="D998" t="s">
+        <v>62</v>
+      </c>
+      <c r="E998" t="s">
+        <v>78</v>
+      </c>
+      <c r="F998" t="s">
+        <v>428</v>
+      </c>
+      <c r="H998">
+        <v>1</v>
+      </c>
+      <c r="J998" s="42">
+        <v>46248</v>
+      </c>
+      <c r="K998" t="s">
+        <v>883</v>
+      </c>
+      <c r="L998" t="s">
+        <v>884</v>
+      </c>
+      <c r="M998" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="999" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A999">
+        <v>468</v>
+      </c>
+      <c r="B999" s="3" t="s">
+        <v>885</v>
+      </c>
+      <c r="C999" s="3" t="s">
+        <v>886</v>
+      </c>
+      <c r="D999" t="s">
+        <v>62</v>
+      </c>
+      <c r="E999" t="s">
+        <v>78</v>
+      </c>
+      <c r="F999" t="s">
+        <v>428</v>
+      </c>
+      <c r="H999">
+        <v>0.5</v>
+      </c>
+      <c r="J999" s="42">
+        <v>46248</v>
+      </c>
+      <c r="K999" t="s">
+        <v>887</v>
+      </c>
+      <c r="L999" t="s">
+        <v>888</v>
+      </c>
+      <c r="M999" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1000" spans="1:13" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A1000">
+        <v>469</v>
+      </c>
+      <c r="B1000" s="3" t="s">
+        <v>889</v>
+      </c>
+      <c r="C1000" s="3" t="s">
+        <v>890</v>
+      </c>
+      <c r="D1000" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1000" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1000" t="s">
+        <v>428</v>
+      </c>
+      <c r="H1000">
+        <v>0.25</v>
+      </c>
+      <c r="J1000" s="42">
+        <v>46248</v>
+      </c>
+      <c r="K1000" t="s">
+        <v>891</v>
+      </c>
+      <c r="L1000" t="s">
+        <v>892</v>
+      </c>
+      <c r="M1000" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1001" spans="1:13" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A1001">
+        <v>470</v>
+      </c>
+      <c r="B1001" s="3" t="s">
+        <v>893</v>
+      </c>
+      <c r="C1001" s="3" t="s">
+        <v>894</v>
+      </c>
+      <c r="D1001" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1001" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1001" t="s">
+        <v>427</v>
+      </c>
+      <c r="H1001">
+        <v>3</v>
+      </c>
+      <c r="J1001" s="42">
+        <v>46248</v>
+      </c>
+      <c r="K1001" t="s">
+        <v>895</v>
+      </c>
+      <c r="L1001" t="s">
+        <v>896</v>
+      </c>
+      <c r="M1001" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1002" spans="1:13" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A1002">
+        <v>471</v>
+      </c>
+      <c r="B1002" s="3" t="s">
+        <v>897</v>
+      </c>
+      <c r="C1002" s="3" t="s">
+        <v>898</v>
+      </c>
+      <c r="D1002" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1002" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1002" t="s">
+        <v>427</v>
+      </c>
+      <c r="H1002">
+        <v>1.5</v>
+      </c>
+      <c r="J1002" s="42">
+        <v>46248</v>
+      </c>
+      <c r="K1002" t="s">
+        <v>899</v>
+      </c>
+      <c r="L1002" t="s">
+        <v>900</v>
+      </c>
+      <c r="M1002" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1003" spans="1:13" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A1003">
+        <v>472</v>
+      </c>
+      <c r="B1003" s="3" t="s">
+        <v>901</v>
+      </c>
+      <c r="C1003" s="3" t="s">
+        <v>902</v>
+      </c>
+      <c r="D1003" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1003" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1003" t="s">
+        <v>431</v>
+      </c>
+      <c r="H1003">
+        <v>0.75</v>
+      </c>
+      <c r="J1003" s="42">
+        <v>46248</v>
+      </c>
+      <c r="K1003" t="s">
+        <v>903</v>
+      </c>
+      <c r="L1003" t="s">
+        <v>904</v>
+      </c>
+      <c r="M1003" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1004" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1004">
+        <v>473</v>
+      </c>
+      <c r="B1004" s="3" t="s">
+        <v>905</v>
+      </c>
+      <c r="C1004" s="3" t="s">
+        <v>906</v>
+      </c>
+      <c r="D1004" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1004" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1004" t="s">
+        <v>431</v>
+      </c>
+      <c r="H1004">
+        <v>0.75</v>
+      </c>
+      <c r="J1004" s="42">
+        <v>46248</v>
+      </c>
+      <c r="K1004" t="s">
+        <v>907</v>
+      </c>
+      <c r="L1004" t="s">
+        <v>908</v>
+      </c>
+      <c r="M1004" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1005" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1005">
+        <v>474</v>
+      </c>
+      <c r="B1005" s="3" t="s">
+        <v>909</v>
+      </c>
+      <c r="C1005" s="3" t="s">
+        <v>910</v>
+      </c>
+      <c r="D1005" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1005" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1005" t="s">
+        <v>428</v>
+      </c>
+      <c r="H1005">
+        <v>0.5</v>
+      </c>
+      <c r="J1005" s="42">
+        <v>46248</v>
+      </c>
+      <c r="K1005" t="s">
+        <v>911</v>
+      </c>
+      <c r="L1005" t="s">
+        <v>912</v>
+      </c>
+      <c r="M1005" t="s">
+        <v>182</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:M273" xr:uid="{00000000-0001-0000-0100-000000000000}">
@@ -18372,26 +18744,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="2e20d828-e3fd-41fd-921c-fbe0ff523ae8">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="adfc7943-f9ee-4478-a01e-ebfcb6e54f53" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100959716F11FB6F9409089B98D1C11D330" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="bc55ac45923017d94ee4534da3224188">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="2e20d828-e3fd-41fd-921c-fbe0ff523ae8" xmlns:ns3="adfc7943-f9ee-4478-a01e-ebfcb6e54f53" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="5bc17ad4f23ab8382a0bb5b03decca58" ns2:_="" ns3:_="">
     <xsd:import namespace="2e20d828-e3fd-41fd-921c-fbe0ff523ae8"/>
@@ -18646,26 +18998,27 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{737DCCA1-99B2-40A5-A4E9-9FBBAC380C60}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{407A8743-A532-48E3-9004-715BF423F4DA}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="2e20d828-e3fd-41fd-921c-fbe0ff523ae8"/>
-    <ds:schemaRef ds:uri="adfc7943-f9ee-4478-a01e-ebfcb6e54f53"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="2e20d828-e3fd-41fd-921c-fbe0ff523ae8">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="adfc7943-f9ee-4478-a01e-ebfcb6e54f53" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5CE6A3B7-F954-4629-B802-2205DECE6851}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -18682,4 +19035,23 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{737DCCA1-99B2-40A5-A4E9-9FBBAC380C60}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{407A8743-A532-48E3-9004-715BF423F4DA}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="2e20d828-e3fd-41fd-921c-fbe0ff523ae8"/>
+    <ds:schemaRef ds:uri="adfc7943-f9ee-4478-a01e-ebfcb6e54f53"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Sync 2026-08-17: 79 Katana tasks reviewed - all existing (#291-#366, #461-#465)
Updates: priority corrections for 29 tasks, status In review for #318/#461/#462,
assignees for #324/#355/#359, notes for 22 tasks.
All GitHub, Monday.com, project_data.json, and Excel updated.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/project_time_sheet.xlsx
+++ b/project_time_sheet.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30228"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{169DDE66-1599-4C9B-93B3-BE14E466E66C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECA09DB0-2BE5-4B4D-9AC2-06A4383CC9A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2524" uniqueCount="913">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2548" uniqueCount="937">
   <si>
     <t xml:space="preserve">  Project Time Sheet — User Guide</t>
   </si>
@@ -2776,6 +2776,78 @@
   </si>
   <si>
     <t>Commit 78d2f08 (17:01). Workflow.md (+20) and ui/docs/content.html (+3).</t>
+  </si>
+  <si>
+    <t>Tested the IPC after updating the bios, ran 3 phantom of 30min, no sign of lagging or getting slow</t>
+  </si>
+  <si>
+    <t>worked well with JM's logic</t>
+  </si>
+  <si>
+    <t>Created a new distribution according to JM's logic and multiple phantom runs proved its evenly distributing the products to robots</t>
+  </si>
+  <si>
+    <t>Consolidation needs time and resources and testing on all the different types of robot cells ABI has</t>
+  </si>
+  <si>
+    <t>Validated the Katana side and the robot side cut points are accurate +/- 3mm</t>
+  </si>
+  <si>
+    <t>Scroll should be removed for the user pages, Katana shouldn't have any scroll page, except information ie. manual user</t>
+  </si>
+  <si>
+    <t>Review the UI</t>
+  </si>
+  <si>
+    <t>come up with a plan for this</t>
+  </si>
+  <si>
+    <t>Need to fix the bug, also should be in English and Spanish only</t>
+  </si>
+  <si>
+    <t>On hold, pending review</t>
+  </si>
+  <si>
+    <t>On hold, pending review || 2026-08-14 KH is working on it</t>
+  </si>
+  <si>
+    <t>Just hide it</t>
+  </si>
+  <si>
+    <t>Pending to review</t>
+  </si>
+  <si>
+    <t>Include deep tank cycles recipe dependant, request Controls. Ask current status of this.</t>
+  </si>
+  <si>
+    <t>DG - started fixing layouts/search; content in .md files, system auto-generates layout. Someone needs to generate correct up-to-date documentation.</t>
+  </si>
+  <si>
+    <t>Ask Controls for make this</t>
+  </si>
+  <si>
+    <t>Export is complete, waiting for controls to finalize the settings</t>
+  </si>
+  <si>
+    <t>Split client access vs ABI</t>
+  </si>
+  <si>
+    <t>be more specific</t>
+  </si>
+  <si>
+    <t>This is already in the 40 item</t>
+  </si>
+  <si>
+    <t>Beckoff IPC reaches &gt;4 GHZ speed; tested with phantom mode and production mode, IPC performed well</t>
+  </si>
+  <si>
+    <t>Require Controls || 2026-08-14 KH is working on it</t>
+  </si>
+  <si>
+    <t>no show</t>
+  </si>
+  <si>
+    <t>no BDF</t>
   </si>
 </sst>
 </file>
@@ -12038,7 +12110,7 @@
         <v>78</v>
       </c>
       <c r="F274" s="164" t="s">
-        <v>431</v>
+        <v>427</v>
       </c>
       <c r="G274" s="164"/>
       <c r="H274" s="164">
@@ -12049,7 +12121,9 @@
       <c r="K274" s="163" t="s">
         <v>661</v>
       </c>
-      <c r="L274" s="163"/>
+      <c r="L274" s="163" t="s">
+        <v>913</v>
+      </c>
       <c r="M274" s="164"/>
       <c r="N274" s="163"/>
     </row>
@@ -12096,7 +12170,7 @@
         <v>78</v>
       </c>
       <c r="F276" s="164" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="G276" s="164"/>
       <c r="H276" s="164"/>
@@ -12105,7 +12179,9 @@
       <c r="K276" s="163" t="s">
         <v>663</v>
       </c>
-      <c r="L276" s="163"/>
+      <c r="L276" s="163" t="s">
+        <v>914</v>
+      </c>
       <c r="M276" s="164"/>
       <c r="N276" s="163"/>
     </row>
@@ -12124,7 +12200,7 @@
         <v>78</v>
       </c>
       <c r="F277" s="164" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="G277" s="164"/>
       <c r="H277" s="164"/>
@@ -12133,7 +12209,9 @@
       <c r="K277" s="163" t="s">
         <v>664</v>
       </c>
-      <c r="L277" s="163"/>
+      <c r="L277" s="163" t="s">
+        <v>915</v>
+      </c>
       <c r="M277" s="164"/>
       <c r="N277" s="163"/>
     </row>
@@ -12151,7 +12229,7 @@
         <v>78</v>
       </c>
       <c r="F278" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="I278" s="42"/>
       <c r="J278" s="42"/>
@@ -12173,13 +12251,16 @@
         <v>71</v>
       </c>
       <c r="F279" t="s">
-        <v>431</v>
+        <v>428</v>
       </c>
       <c r="I279" s="42"/>
       <c r="J279" s="42"/>
       <c r="K279" t="s">
         <v>666</v>
       </c>
+      <c r="L279" t="s">
+        <v>916</v>
+      </c>
     </row>
     <row r="280" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B280" s="3" t="s">
@@ -12192,13 +12273,16 @@
         <v>78</v>
       </c>
       <c r="F280" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="I280" s="42"/>
       <c r="J280" s="42"/>
       <c r="K280" t="s">
         <v>415</v>
       </c>
+      <c r="L280" t="s">
+        <v>917</v>
+      </c>
     </row>
     <row r="281" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B281" s="3" t="s">
@@ -12211,7 +12295,7 @@
         <v>78</v>
       </c>
       <c r="F281" t="s">
-        <v>431</v>
+        <v>427</v>
       </c>
       <c r="I281" s="42"/>
       <c r="J281" s="42"/>
@@ -12233,7 +12317,7 @@
         <v>78</v>
       </c>
       <c r="F282" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="I282" s="42"/>
       <c r="J282" s="42"/>
@@ -12255,7 +12339,7 @@
         <v>78</v>
       </c>
       <c r="F283" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="I283" s="42"/>
       <c r="J283" s="42"/>
@@ -12277,7 +12361,7 @@
         <v>68</v>
       </c>
       <c r="F284" t="s">
-        <v>427</v>
+        <v>431</v>
       </c>
       <c r="I284" s="42"/>
       <c r="J284" s="42"/>
@@ -12311,6 +12395,9 @@
       <c r="K285" t="s">
         <v>670</v>
       </c>
+      <c r="L285" t="s">
+        <v>918</v>
+      </c>
     </row>
     <row r="286" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B286" s="3" t="s">
@@ -12330,6 +12417,9 @@
       <c r="K286" t="s">
         <v>671</v>
       </c>
+      <c r="L286" t="s">
+        <v>919</v>
+      </c>
     </row>
     <row r="287" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B287" s="3" t="s">
@@ -12377,7 +12467,7 @@
         <v>673</v>
       </c>
     </row>
-    <row r="289" spans="2:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="289" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B289" s="3" t="s">
         <v>360</v>
       </c>
@@ -12402,7 +12492,7 @@
         <v>674</v>
       </c>
     </row>
-    <row r="290" spans="2:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="290" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B290" s="3" t="s">
         <v>361</v>
       </c>
@@ -12423,8 +12513,11 @@
       <c r="K290" t="s">
         <v>675</v>
       </c>
-    </row>
-    <row r="291" spans="2:11" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="L290" t="s">
+        <v>920</v>
+      </c>
+    </row>
+    <row r="291" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B291" s="3" t="s">
         <v>362</v>
       </c>
@@ -12438,7 +12531,7 @@
         <v>71</v>
       </c>
       <c r="F291" t="s">
-        <v>431</v>
+        <v>428</v>
       </c>
       <c r="I291" s="42"/>
       <c r="J291" s="42"/>
@@ -12446,7 +12539,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="292" spans="2:11" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="292" spans="2:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B292" s="3" t="s">
         <v>363</v>
       </c>
@@ -12470,8 +12563,11 @@
       <c r="K292" t="s">
         <v>676</v>
       </c>
-    </row>
-    <row r="293" spans="2:11" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="L292" t="s">
+        <v>921</v>
+      </c>
+    </row>
+    <row r="293" spans="2:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B293" s="3" t="s">
         <v>364</v>
       </c>
@@ -12493,7 +12589,7 @@
         <v>677</v>
       </c>
     </row>
-    <row r="294" spans="2:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="294" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B294" s="3" t="s">
         <v>365</v>
       </c>
@@ -12514,8 +12610,11 @@
       <c r="K294" t="s">
         <v>416</v>
       </c>
-    </row>
-    <row r="295" spans="2:11" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="L294" t="s">
+        <v>922</v>
+      </c>
+    </row>
+    <row r="295" spans="2:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B295" s="3" t="s">
         <v>366</v>
       </c>
@@ -12536,8 +12635,11 @@
       <c r="K295" t="s">
         <v>678</v>
       </c>
-    </row>
-    <row r="296" spans="2:11" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="L295" t="s">
+        <v>923</v>
+      </c>
+    </row>
+    <row r="296" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B296" s="3" t="s">
         <v>367</v>
       </c>
@@ -12562,7 +12664,7 @@
         <v>679</v>
       </c>
     </row>
-    <row r="297" spans="2:11" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="297" spans="2:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B297" s="3" t="s">
         <v>368</v>
       </c>
@@ -12587,7 +12689,7 @@
         <v>680</v>
       </c>
     </row>
-    <row r="298" spans="2:11" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="298" spans="2:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B298" s="3" t="s">
         <v>369</v>
       </c>
@@ -12601,7 +12703,7 @@
         <v>68</v>
       </c>
       <c r="F298" t="s">
-        <v>431</v>
+        <v>427</v>
       </c>
       <c r="H298">
         <v>6</v>
@@ -12614,7 +12716,7 @@
         <v>681</v>
       </c>
     </row>
-    <row r="299" spans="2:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="299" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B299" s="3" t="s">
         <v>370</v>
       </c>
@@ -12636,7 +12738,7 @@
         <v>682</v>
       </c>
     </row>
-    <row r="300" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="300" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B300" s="3" t="s">
         <v>371</v>
       </c>
@@ -12661,7 +12763,7 @@
         <v>683</v>
       </c>
     </row>
-    <row r="301" spans="2:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="301" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B301" s="3" t="s">
         <v>372</v>
       </c>
@@ -12669,7 +12771,7 @@
         <v>607</v>
       </c>
       <c r="E301" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="F301" t="s">
         <v>431</v>
@@ -12680,7 +12782,7 @@
         <v>417</v>
       </c>
     </row>
-    <row r="302" spans="2:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="302" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B302" s="3" t="s">
         <v>373</v>
       </c>
@@ -12694,7 +12796,7 @@
         <v>71</v>
       </c>
       <c r="F302" t="s">
-        <v>431</v>
+        <v>428</v>
       </c>
       <c r="H302">
         <v>2</v>
@@ -12705,7 +12807,7 @@
         <v>683</v>
       </c>
     </row>
-    <row r="303" spans="2:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="303" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B303" s="3" t="s">
         <v>374</v>
       </c>
@@ -12716,7 +12818,7 @@
         <v>71</v>
       </c>
       <c r="F303" t="s">
-        <v>431</v>
+        <v>428</v>
       </c>
       <c r="I303" s="42"/>
       <c r="J303" s="42"/>
@@ -12724,7 +12826,7 @@
         <v>684</v>
       </c>
     </row>
-    <row r="304" spans="2:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="304" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B304" s="3" t="s">
         <v>375</v>
       </c>
@@ -12746,7 +12848,7 @@
         <v>685</v>
       </c>
     </row>
-    <row r="305" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="305" spans="2:12" ht="57.6" x14ac:dyDescent="0.3">
       <c r="B305" s="3" t="s">
         <v>376</v>
       </c>
@@ -12760,7 +12862,7 @@
         <v>68</v>
       </c>
       <c r="F305" t="s">
-        <v>431</v>
+        <v>427</v>
       </c>
       <c r="I305" s="42"/>
       <c r="J305" s="42"/>
@@ -12768,7 +12870,7 @@
         <v>686</v>
       </c>
     </row>
-    <row r="306" spans="2:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="306" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B306" s="3" t="s">
         <v>377</v>
       </c>
@@ -12793,7 +12895,7 @@
         <v>683</v>
       </c>
     </row>
-    <row r="307" spans="2:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="307" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B307" s="3" t="s">
         <v>378</v>
       </c>
@@ -12815,7 +12917,7 @@
         <v>687</v>
       </c>
     </row>
-    <row r="308" spans="2:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="308" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B308" s="3" t="s">
         <v>379</v>
       </c>
@@ -12826,7 +12928,7 @@
         <v>71</v>
       </c>
       <c r="F308" t="s">
-        <v>431</v>
+        <v>428</v>
       </c>
       <c r="I308" s="42"/>
       <c r="J308" s="42"/>
@@ -12834,7 +12936,7 @@
         <v>688</v>
       </c>
     </row>
-    <row r="309" spans="2:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="309" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B309" s="3" t="s">
         <v>380</v>
       </c>
@@ -12848,7 +12950,7 @@
         <v>71</v>
       </c>
       <c r="F309" t="s">
-        <v>431</v>
+        <v>428</v>
       </c>
       <c r="I309" s="42"/>
       <c r="J309" s="42"/>
@@ -12856,7 +12958,7 @@
         <v>688</v>
       </c>
     </row>
-    <row r="310" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="310" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B310" s="3" t="s">
         <v>381</v>
       </c>
@@ -12882,8 +12984,11 @@
       <c r="K310" t="s">
         <v>683</v>
       </c>
-    </row>
-    <row r="311" spans="2:11" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="L310" t="s">
+        <v>924</v>
+      </c>
+    </row>
+    <row r="311" spans="2:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B311" s="3" t="s">
         <v>382</v>
       </c>
@@ -12905,7 +13010,7 @@
         <v>688</v>
       </c>
     </row>
-    <row r="312" spans="2:11" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="312" spans="2:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B312" s="3" t="s">
         <v>383</v>
       </c>
@@ -12930,7 +13035,7 @@
         <v>683</v>
       </c>
     </row>
-    <row r="313" spans="2:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="313" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B313" s="3" t="s">
         <v>384</v>
       </c>
@@ -12952,7 +13057,7 @@
         <v>685</v>
       </c>
     </row>
-    <row r="314" spans="2:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="314" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B314" s="3" t="s">
         <v>385</v>
       </c>
@@ -12977,7 +13082,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="315" spans="2:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="315" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B315" s="3" t="s">
         <v>386</v>
       </c>
@@ -12999,7 +13104,7 @@
         <v>688</v>
       </c>
     </row>
-    <row r="316" spans="2:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="316" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B316" s="3" t="s">
         <v>387</v>
       </c>
@@ -13024,7 +13129,7 @@
         <v>690</v>
       </c>
     </row>
-    <row r="317" spans="2:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="317" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B317" s="3" t="s">
         <v>388</v>
       </c>
@@ -13049,7 +13154,7 @@
         <v>690</v>
       </c>
     </row>
-    <row r="318" spans="2:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="318" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B318" s="3" t="s">
         <v>389</v>
       </c>
@@ -13070,8 +13175,11 @@
       <c r="K318" t="s">
         <v>688</v>
       </c>
-    </row>
-    <row r="319" spans="2:11" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="L318" t="s">
+        <v>925</v>
+      </c>
+    </row>
+    <row r="319" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B319" s="3" t="s">
         <v>390</v>
       </c>
@@ -13082,7 +13190,7 @@
         <v>71</v>
       </c>
       <c r="F319" t="s">
-        <v>431</v>
+        <v>428</v>
       </c>
       <c r="I319" s="42"/>
       <c r="J319" s="42"/>
@@ -13090,7 +13198,7 @@
         <v>688</v>
       </c>
     </row>
-    <row r="320" spans="2:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="320" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B320" s="3" t="s">
         <v>391</v>
       </c>
@@ -13104,15 +13212,18 @@
         <v>71</v>
       </c>
       <c r="F320" t="s">
-        <v>431</v>
+        <v>428</v>
       </c>
       <c r="I320" s="42"/>
       <c r="J320" s="42"/>
       <c r="K320" t="s">
         <v>688</v>
       </c>
-    </row>
-    <row r="321" spans="2:11" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="L320" t="s">
+        <v>926</v>
+      </c>
+    </row>
+    <row r="321" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B321" s="3" t="s">
         <v>392</v>
       </c>
@@ -13139,7 +13250,7 @@
         <v>683</v>
       </c>
     </row>
-    <row r="322" spans="2:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="322" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B322" s="3" t="s">
         <v>393</v>
       </c>
@@ -13163,8 +13274,11 @@
       <c r="K322" t="s">
         <v>689</v>
       </c>
-    </row>
-    <row r="323" spans="2:11" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="L322" t="s">
+        <v>927</v>
+      </c>
+    </row>
+    <row r="323" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B323" s="3" t="s">
         <v>394</v>
       </c>
@@ -13178,7 +13292,7 @@
         <v>71</v>
       </c>
       <c r="F323" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="I323" s="42"/>
       <c r="J323" s="42"/>
@@ -13186,7 +13300,7 @@
         <v>688</v>
       </c>
     </row>
-    <row r="324" spans="2:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="324" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B324" s="3" t="s">
         <v>395</v>
       </c>
@@ -13205,7 +13319,7 @@
         <v>417</v>
       </c>
     </row>
-    <row r="325" spans="2:11" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="325" spans="2:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B325" s="3" t="s">
         <v>396</v>
       </c>
@@ -13226,8 +13340,11 @@
       <c r="K325" t="s">
         <v>418</v>
       </c>
-    </row>
-    <row r="326" spans="2:11" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="L325" t="s">
+        <v>928</v>
+      </c>
+    </row>
+    <row r="326" spans="2:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B326" s="3" t="s">
         <v>397</v>
       </c>
@@ -13241,15 +13358,18 @@
         <v>71</v>
       </c>
       <c r="F326" t="s">
-        <v>431</v>
+        <v>428</v>
       </c>
       <c r="I326" s="42"/>
       <c r="J326" s="42"/>
       <c r="K326" t="s">
         <v>691</v>
       </c>
-    </row>
-    <row r="327" spans="2:11" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="L326" t="s">
+        <v>929</v>
+      </c>
+    </row>
+    <row r="327" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B327" s="3" t="s">
         <v>398</v>
       </c>
@@ -13268,7 +13388,7 @@
         <v>692</v>
       </c>
     </row>
-    <row r="328" spans="2:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="328" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B328" s="3" t="s">
         <v>399</v>
       </c>
@@ -13290,7 +13410,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="329" spans="2:11" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="329" spans="2:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B329" s="3" t="s">
         <v>400</v>
       </c>
@@ -13312,7 +13432,7 @@
         <v>692</v>
       </c>
     </row>
-    <row r="330" spans="2:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="330" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B330" s="3" t="s">
         <v>401</v>
       </c>
@@ -13326,15 +13446,18 @@
         <v>78</v>
       </c>
       <c r="F330" t="s">
-        <v>431</v>
+        <v>428</v>
       </c>
       <c r="I330" s="42"/>
       <c r="J330" s="42"/>
       <c r="K330" t="s">
         <v>693</v>
       </c>
-    </row>
-    <row r="331" spans="2:11" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="L330" t="s">
+        <v>930</v>
+      </c>
+    </row>
+    <row r="331" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B331" s="3" t="s">
         <v>402</v>
       </c>
@@ -13355,8 +13478,11 @@
       <c r="K331" t="s">
         <v>694</v>
       </c>
-    </row>
-    <row r="332" spans="2:11" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="L331" t="s">
+        <v>931</v>
+      </c>
+    </row>
+    <row r="332" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B332" s="3" t="s">
         <v>403</v>
       </c>
@@ -13378,7 +13504,7 @@
         <v>695</v>
       </c>
     </row>
-    <row r="333" spans="2:11" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="333" spans="2:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B333" s="3" t="s">
         <v>404</v>
       </c>
@@ -13392,7 +13518,7 @@
         <v>71</v>
       </c>
       <c r="F333" t="s">
-        <v>431</v>
+        <v>428</v>
       </c>
       <c r="I333" s="42"/>
       <c r="J333" s="42"/>
@@ -13400,7 +13526,7 @@
         <v>696</v>
       </c>
     </row>
-    <row r="334" spans="2:11" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="334" spans="2:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B334" s="3" t="s">
         <v>405</v>
       </c>
@@ -13414,7 +13540,7 @@
         <v>71</v>
       </c>
       <c r="F334" t="s">
-        <v>431</v>
+        <v>428</v>
       </c>
       <c r="I334" s="42"/>
       <c r="J334" s="42"/>
@@ -13422,7 +13548,7 @@
         <v>696</v>
       </c>
     </row>
-    <row r="335" spans="2:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="335" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B335" s="3" t="s">
         <v>406</v>
       </c>
@@ -13436,7 +13562,7 @@
         <v>71</v>
       </c>
       <c r="F335" t="s">
-        <v>431</v>
+        <v>428</v>
       </c>
       <c r="I335" s="42"/>
       <c r="J335" s="42"/>
@@ -13444,7 +13570,7 @@
         <v>696</v>
       </c>
     </row>
-    <row r="336" spans="2:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="336" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B336" s="3" t="s">
         <v>407</v>
       </c>
@@ -13529,7 +13655,7 @@
         <v>78</v>
       </c>
       <c r="F339" t="s">
-        <v>431</v>
+        <v>428</v>
       </c>
       <c r="H339">
         <v>10</v>
@@ -13570,13 +13696,16 @@
         <v>71</v>
       </c>
       <c r="F341" t="s">
-        <v>431</v>
+        <v>428</v>
       </c>
       <c r="I341" s="42"/>
       <c r="J341" s="42"/>
       <c r="K341" t="s">
         <v>700</v>
       </c>
+      <c r="L341" t="s">
+        <v>932</v>
+      </c>
     </row>
     <row r="342" spans="2:13" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B342" s="3" t="s">
@@ -13586,7 +13715,7 @@
         <v>648</v>
       </c>
       <c r="D342" t="s">
-        <v>61</v>
+        <v>655</v>
       </c>
       <c r="E342" t="s">
         <v>78</v>
@@ -13602,6 +13731,9 @@
       <c r="K342" t="s">
         <v>701</v>
       </c>
+      <c r="L342" t="s">
+        <v>933</v>
+      </c>
     </row>
     <row r="343" spans="2:13" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B343" s="3" t="s">
@@ -13614,7 +13746,7 @@
         <v>71</v>
       </c>
       <c r="F343" t="s">
-        <v>427</v>
+        <v>431</v>
       </c>
       <c r="I343" s="42"/>
       <c r="J343" s="42"/>
@@ -13636,7 +13768,7 @@
         <v>71</v>
       </c>
       <c r="F344" t="s">
-        <v>431</v>
+        <v>428</v>
       </c>
       <c r="I344" s="42"/>
       <c r="J344" s="42"/>
@@ -13736,6 +13868,9 @@
       <c r="K348" t="s">
         <v>703</v>
       </c>
+      <c r="L348" t="s">
+        <v>934</v>
+      </c>
     </row>
     <row r="349" spans="2:13" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B349" s="3" t="s">
@@ -13755,6 +13890,9 @@
       <c r="K349" t="s">
         <v>704</v>
       </c>
+      <c r="L349" t="s">
+        <v>935</v>
+      </c>
     </row>
     <row r="350" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B350" s="3" t="s">
@@ -16026,7 +16164,7 @@
         <v>870</v>
       </c>
       <c r="E444" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="F444" t="s">
         <v>428</v>
@@ -16053,7 +16191,7 @@
         <v>873</v>
       </c>
       <c r="E445" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="F445" t="s">
         <v>428</v>
@@ -16137,6 +16275,9 @@
       <c r="J448" s="42"/>
       <c r="K448" t="s">
         <v>871</v>
+      </c>
+      <c r="L448" t="s">
+        <v>936</v>
       </c>
       <c r="M448" t="s">
         <v>69</v>

</xml_diff>

<commit_message>
Add 15 new Eye-Q tasks (#475-#489): ABI.Unity issues #1026-#1040
GitHub issues created with Status=Done, Scope=Eye-Q, Estimates set.
Monday.com subitems created under Eye-Q parent (11002499253).
task_mapping.json: 474 -> 489 entries.
project_data.json: 455 -> 470 tasks.
project_time_sheet.xlsx: rows 1006-1020 added.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/project_time_sheet.xlsx
+++ b/project_time_sheet.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30228"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECA09DB0-2BE5-4B4D-9AC2-06A4383CC9A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9C85290-57EC-41E4-9212-66FDB17DC545}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2548" uniqueCount="937">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2653" uniqueCount="982">
   <si>
     <t xml:space="preserve">  Project Time Sheet — User Guide</t>
   </si>
@@ -2848,6 +2848,141 @@
   </si>
   <si>
     <t>no BDF</t>
+  </si>
+  <si>
+    <t>Tablet and touch-friendly workflow UI</t>
+  </si>
+  <si>
+    <t>Improved tablet layouts, touch targets, node dragging, connector interaction, responsive shell behavior, and workflow documentation for coarse-pointer devices.</t>
+  </si>
+  <si>
+    <t>Implemented and committed as ad6fb7b; includes workflow, Train, shell, and documentation updates</t>
+  </si>
+  <si>
+    <t>Pan cavity detection workflow node</t>
+  </si>
+  <si>
+    <t>Added a reusable cavity-detection library and Workflow node that classifies configured pan cavities as occupied or empty and exposes structured results.</t>
+  </si>
+  <si>
+    <t>Implemented and committed as 9c95489; includes detector and workflow-node tests</t>
+  </si>
+  <si>
+    <t>Pan cavity auto-detection and optimization</t>
+  </si>
+  <si>
+    <t>Added automatic cavity-layout detection, workflow API support, UI action, improved detector logic, result handling, tests, and documentation.</t>
+  </si>
+  <si>
+    <t>Implemented and committed as ebe01a1; optimized beyond original fixed R7-6 configuration</t>
+  </si>
+  <si>
+    <t>OpenSpec project integration</t>
+  </si>
+  <si>
+    <t>Added OpenSpec configuration, change-management skills, and command workflows for proposing, applying, updating, syncing, and archiving specifications.</t>
+  </si>
+  <si>
+    <t>Implemented and committed as 8f83217; structured specification-driven development support</t>
+  </si>
+  <si>
+    <t>Experimental synthetic-data feature</t>
+  </si>
+  <si>
+    <t>Integrated the local bakery synthetic-data system with training UI, APIs, engine, dataset handling, configuration, tests, documentation, and an OpenSpec change package.</t>
+  </si>
+  <si>
+    <t>Experimental and rollback-ready; committed as 5ebe7b4</t>
+  </si>
+  <si>
+    <t>Project-aware AI Agent page</t>
+  </si>
+  <si>
+    <t>Created an Agent page with operator and developer profiles, provider routing, guarded project context, image-capable conversation UI, server routes, tests, and documentation.</t>
+  </si>
+  <si>
+    <t>Implemented and committed as 4b97a77; includes prompt-injection boundaries and profile authorization</t>
+  </si>
+  <si>
+    <t>AI Agent usability and configuration</t>
+  </si>
+  <si>
+    <t>Added safe Markdown rendering, Enter-to-send, automatic conversation scrolling, general Settings integration for profile/provider/model, local Ollama support, and developer-mode controls.</t>
+  </si>
+  <si>
+    <t>Implemented and committed as 9816d62; provider configuration centralized in Settings</t>
+  </si>
+  <si>
+    <t>Distinct Agent navigation icon</t>
+  </si>
+  <si>
+    <t>Replaced the duplicated Documentation icon with a dedicated Agent menu icon.</t>
+  </si>
+  <si>
+    <t>Implemented and committed as c8da67d</t>
+  </si>
+  <si>
+    <t>Multi-camera Racer2 workflow support</t>
+  </si>
+  <si>
+    <t>Extended workflow camera-source handling and associated UI behavior for multiple Racer2 cameras, matching the existing multi-camera Ace workflow model.</t>
+  </si>
+  <si>
+    <t>Implemented and committed as abd9f24; includes responsive UI and regression tests</t>
+  </si>
+  <si>
+    <t>Phone tablet and webcam image capture</t>
+  </si>
+  <si>
+    <t>Added file selection, native phone/tablet camera capture, and live webcam capture to the Workflow Upload Image node.</t>
+  </si>
+  <si>
+    <t>Implemented within commit abd9f24 and workflow UI tests</t>
+  </si>
+  <si>
+    <t>Browser camera as a live Workflow source</t>
+  </si>
+  <si>
+    <t>Added Browser camera to the Live Camera node with device preview, single-frame execution, continuous processing, stop behavior, and browser-frame forwarding through the workflow API.</t>
+  </si>
+  <si>
+    <t>Implemented and committed as 0dfacb0; live network camera requires HTTPS on tablets</t>
+  </si>
+  <si>
+    <t>Collapsible Settings groups</t>
+  </si>
+  <si>
+    <t>Converted every generated Settings section into an independently collapsible touch-friendly panel while preserving collapsed state across re-rendering.</t>
+  </si>
+  <si>
+    <t>Implemented and committed as d309b76 with UI regression coverage</t>
+  </si>
+  <si>
+    <t>Descriptions for every setting</t>
+  </si>
+  <si>
+    <t>Added a short explanatory line to every Settings entry, using authored catalog notes where available and readable generated descriptions otherwise.</t>
+  </si>
+  <si>
+    <t>Implemented and committed as d309b76; range, allowed-value, source, lock notes remain separate</t>
+  </si>
+  <si>
+    <t>Installable tablet Progressive Web App</t>
+  </si>
+  <si>
+    <t>Added the web-app manifest, ABI application icons, Apple home-screen metadata, service worker, install controls, standalone landscape behavior, and deterministic icon generation.</t>
+  </si>
+  <si>
+    <t>Implemented and committed as b2ea7dc; live APIs remain network-first</t>
+  </si>
+  <si>
+    <t>iPad status-bar overlap and fullscreen behavior</t>
+  </si>
+  <si>
+    <t>Changed the Apple status-bar presentation, corrected toolbar/sidebar/content safe-area geometry, and added a user-initiated tablet fullscreen control where supported.</t>
+  </si>
+  <si>
+    <t>Implemented and committed as b2ea7dc; iPadOS does not permit PWA to hide system indicators automatically</t>
   </si>
 </sst>
 </file>
@@ -4729,7 +4864,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:N1005"/>
+  <dimension ref="A1:N1020"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="7.6640625" customWidth="1"/>
@@ -18756,6 +18891,486 @@
         <v>912</v>
       </c>
       <c r="M1005" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1006" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1006">
+        <v>475</v>
+      </c>
+      <c r="B1006" s="3" t="s">
+        <v>937</v>
+      </c>
+      <c r="C1006" s="3" t="s">
+        <v>938</v>
+      </c>
+      <c r="D1006" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1006" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1006" t="s">
+        <v>427</v>
+      </c>
+      <c r="H1006">
+        <v>6</v>
+      </c>
+      <c r="J1006" s="42">
+        <v>46251</v>
+      </c>
+      <c r="L1006" t="s">
+        <v>939</v>
+      </c>
+      <c r="M1006" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1007" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1007">
+        <v>476</v>
+      </c>
+      <c r="B1007" s="3" t="s">
+        <v>940</v>
+      </c>
+      <c r="C1007" s="3" t="s">
+        <v>941</v>
+      </c>
+      <c r="D1007" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1007" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1007" t="s">
+        <v>427</v>
+      </c>
+      <c r="H1007">
+        <v>6</v>
+      </c>
+      <c r="J1007" s="42">
+        <v>46251</v>
+      </c>
+      <c r="L1007" t="s">
+        <v>942</v>
+      </c>
+      <c r="M1007" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1008" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1008">
+        <v>477</v>
+      </c>
+      <c r="B1008" s="3" t="s">
+        <v>943</v>
+      </c>
+      <c r="C1008" s="3" t="s">
+        <v>944</v>
+      </c>
+      <c r="D1008" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1008" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1008" t="s">
+        <v>427</v>
+      </c>
+      <c r="H1008">
+        <v>6</v>
+      </c>
+      <c r="J1008" s="42">
+        <v>46251</v>
+      </c>
+      <c r="L1008" t="s">
+        <v>945</v>
+      </c>
+      <c r="M1008" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1009" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1009">
+        <v>478</v>
+      </c>
+      <c r="B1009" s="3" t="s">
+        <v>946</v>
+      </c>
+      <c r="C1009" s="3" t="s">
+        <v>947</v>
+      </c>
+      <c r="D1009" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1009" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1009" t="s">
+        <v>431</v>
+      </c>
+      <c r="H1009">
+        <v>3</v>
+      </c>
+      <c r="J1009" s="42">
+        <v>46251</v>
+      </c>
+      <c r="L1009" t="s">
+        <v>948</v>
+      </c>
+      <c r="M1009" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1010" spans="1:13" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A1010">
+        <v>479</v>
+      </c>
+      <c r="B1010" s="3" t="s">
+        <v>949</v>
+      </c>
+      <c r="C1010" s="3" t="s">
+        <v>950</v>
+      </c>
+      <c r="D1010" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1010" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1010" t="s">
+        <v>431</v>
+      </c>
+      <c r="H1010">
+        <v>8</v>
+      </c>
+      <c r="J1010" s="42">
+        <v>46251</v>
+      </c>
+      <c r="L1010" t="s">
+        <v>951</v>
+      </c>
+      <c r="M1010" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1011" spans="1:13" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A1011">
+        <v>480</v>
+      </c>
+      <c r="B1011" s="3" t="s">
+        <v>952</v>
+      </c>
+      <c r="C1011" s="3" t="s">
+        <v>953</v>
+      </c>
+      <c r="D1011" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1011" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1011" t="s">
+        <v>427</v>
+      </c>
+      <c r="H1011">
+        <v>10</v>
+      </c>
+      <c r="J1011" s="42">
+        <v>46251</v>
+      </c>
+      <c r="L1011" t="s">
+        <v>954</v>
+      </c>
+      <c r="M1011" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1012" spans="1:13" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A1012">
+        <v>481</v>
+      </c>
+      <c r="B1012" s="3" t="s">
+        <v>955</v>
+      </c>
+      <c r="C1012" s="3" t="s">
+        <v>956</v>
+      </c>
+      <c r="D1012" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1012" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1012" t="s">
+        <v>427</v>
+      </c>
+      <c r="H1012">
+        <v>5</v>
+      </c>
+      <c r="J1012" s="42">
+        <v>46251</v>
+      </c>
+      <c r="L1012" t="s">
+        <v>957</v>
+      </c>
+      <c r="M1012" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1013" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A1013">
+        <v>482</v>
+      </c>
+      <c r="B1013" s="3" t="s">
+        <v>958</v>
+      </c>
+      <c r="C1013" s="3" t="s">
+        <v>959</v>
+      </c>
+      <c r="D1013" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1013" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1013" t="s">
+        <v>428</v>
+      </c>
+      <c r="H1013">
+        <v>0.5</v>
+      </c>
+      <c r="J1013" s="42">
+        <v>46251</v>
+      </c>
+      <c r="L1013" t="s">
+        <v>960</v>
+      </c>
+      <c r="M1013" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1014" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1014">
+        <v>483</v>
+      </c>
+      <c r="B1014" s="3" t="s">
+        <v>961</v>
+      </c>
+      <c r="C1014" s="3" t="s">
+        <v>962</v>
+      </c>
+      <c r="D1014" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1014" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1014" t="s">
+        <v>427</v>
+      </c>
+      <c r="H1014">
+        <v>5</v>
+      </c>
+      <c r="J1014" s="42">
+        <v>46251</v>
+      </c>
+      <c r="L1014" t="s">
+        <v>963</v>
+      </c>
+      <c r="M1014" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1015" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1015">
+        <v>484</v>
+      </c>
+      <c r="B1015" s="3" t="s">
+        <v>964</v>
+      </c>
+      <c r="C1015" s="3" t="s">
+        <v>965</v>
+      </c>
+      <c r="D1015" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1015" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1015" t="s">
+        <v>427</v>
+      </c>
+      <c r="H1015">
+        <v>3</v>
+      </c>
+      <c r="J1015" s="42">
+        <v>46251</v>
+      </c>
+      <c r="L1015" t="s">
+        <v>966</v>
+      </c>
+      <c r="M1015" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1016" spans="1:13" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A1016">
+        <v>485</v>
+      </c>
+      <c r="B1016" s="3" t="s">
+        <v>967</v>
+      </c>
+      <c r="C1016" s="3" t="s">
+        <v>968</v>
+      </c>
+      <c r="D1016" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1016" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1016" t="s">
+        <v>427</v>
+      </c>
+      <c r="H1016">
+        <v>5</v>
+      </c>
+      <c r="J1016" s="42">
+        <v>46251</v>
+      </c>
+      <c r="L1016" t="s">
+        <v>969</v>
+      </c>
+      <c r="M1016" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1017" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1017">
+        <v>486</v>
+      </c>
+      <c r="B1017" s="3" t="s">
+        <v>970</v>
+      </c>
+      <c r="C1017" s="3" t="s">
+        <v>971</v>
+      </c>
+      <c r="D1017" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1017" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1017" t="s">
+        <v>428</v>
+      </c>
+      <c r="H1017">
+        <v>2</v>
+      </c>
+      <c r="J1017" s="42">
+        <v>46251</v>
+      </c>
+      <c r="L1017" t="s">
+        <v>972</v>
+      </c>
+      <c r="M1017" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1018" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1018">
+        <v>487</v>
+      </c>
+      <c r="B1018" s="3" t="s">
+        <v>973</v>
+      </c>
+      <c r="C1018" s="3" t="s">
+        <v>974</v>
+      </c>
+      <c r="D1018" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1018" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1018" t="s">
+        <v>428</v>
+      </c>
+      <c r="H1018">
+        <v>2</v>
+      </c>
+      <c r="J1018" s="42">
+        <v>46251</v>
+      </c>
+      <c r="L1018" t="s">
+        <v>975</v>
+      </c>
+      <c r="M1018" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1019" spans="1:13" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A1019">
+        <v>488</v>
+      </c>
+      <c r="B1019" s="3" t="s">
+        <v>976</v>
+      </c>
+      <c r="C1019" s="3" t="s">
+        <v>977</v>
+      </c>
+      <c r="D1019" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1019" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1019" t="s">
+        <v>427</v>
+      </c>
+      <c r="H1019">
+        <v>6</v>
+      </c>
+      <c r="J1019" s="42">
+        <v>46251</v>
+      </c>
+      <c r="L1019" t="s">
+        <v>978</v>
+      </c>
+      <c r="M1019" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1020" spans="1:13" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A1020">
+        <v>489</v>
+      </c>
+      <c r="B1020" s="3" t="s">
+        <v>979</v>
+      </c>
+      <c r="C1020" s="3" t="s">
+        <v>980</v>
+      </c>
+      <c r="D1020" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1020" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1020" t="s">
+        <v>431</v>
+      </c>
+      <c r="H1020">
+        <v>3</v>
+      </c>
+      <c r="J1020" s="42">
+        <v>46251</v>
+      </c>
+      <c r="L1020" t="s">
+        <v>981</v>
+      </c>
+      <c r="M1020" t="s">
         <v>182</v>
       </c>
     </row>
@@ -18885,6 +19500,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100959716F11FB6F9409089B98D1C11D330" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="bc55ac45923017d94ee4534da3224188">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="2e20d828-e3fd-41fd-921c-fbe0ff523ae8" xmlns:ns3="adfc7943-f9ee-4478-a01e-ebfcb6e54f53" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="5bc17ad4f23ab8382a0bb5b03decca58" ns2:_="" ns3:_="">
     <xsd:import namespace="2e20d828-e3fd-41fd-921c-fbe0ff523ae8"/>
@@ -19139,15 +19763,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -19160,6 +19775,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{737DCCA1-99B2-40A5-A4E9-9FBBAC380C60}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5CE6A3B7-F954-4629-B802-2205DECE6851}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -19178,14 +19801,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{737DCCA1-99B2-40A5-A4E9-9FBBAC380C60}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{407A8743-A532-48E3-9004-715BF423F4DA}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
Sync 2026-08-18: 79 Katana tasks reviewed (#291-#366, #461-#465)
Status updates (16 tasks): #301,302,306,314,315,317,322,327,329,330,331,339,354,462 -> Done; #316 -> In review; #345 -> In progress.
Target dates added (8 tasks): #302,304,315,327,338,354,365,461.
Scope=Katana set on 74 previously unscoped tasks (#291-#366 excl. #360-#364, #461-#465).
project_data.json: 72 tasks updated.
project_time_sheet.xlsx: 76 rows updated.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/project_time_sheet.xlsx
+++ b/project_time_sheet.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30228"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9C85290-57EC-41E4-9212-66FDB17DC545}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B052D40-1573-4692-A87F-0EE66AEB1929}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2653" uniqueCount="982">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2723" uniqueCount="982">
   <si>
     <t xml:space="preserve">  Project Time Sheet — User Guide</t>
   </si>
@@ -12259,7 +12259,9 @@
       <c r="L274" s="163" t="s">
         <v>913</v>
       </c>
-      <c r="M274" s="164"/>
+      <c r="M274" s="164" t="s">
+        <v>69</v>
+      </c>
       <c r="N274" s="163"/>
     </row>
     <row r="275" spans="1:14" x14ac:dyDescent="0.3">
@@ -12317,7 +12319,9 @@
       <c r="L276" s="163" t="s">
         <v>914</v>
       </c>
-      <c r="M276" s="164"/>
+      <c r="M276" s="164" t="s">
+        <v>69</v>
+      </c>
       <c r="N276" s="163"/>
     </row>
     <row r="277" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -12347,7 +12351,9 @@
       <c r="L277" s="163" t="s">
         <v>915</v>
       </c>
-      <c r="M277" s="164"/>
+      <c r="M277" s="164" t="s">
+        <v>69</v>
+      </c>
       <c r="N277" s="163"/>
     </row>
     <row r="278" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
@@ -12371,6 +12377,9 @@
       <c r="K278" t="s">
         <v>665</v>
       </c>
+      <c r="M278" t="s">
+        <v>69</v>
+      </c>
     </row>
     <row r="279" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
       <c r="B279" s="3" t="s">
@@ -12396,6 +12405,9 @@
       <c r="L279" t="s">
         <v>916</v>
       </c>
+      <c r="M279" t="s">
+        <v>69</v>
+      </c>
     </row>
     <row r="280" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B280" s="3" t="s">
@@ -12418,6 +12430,9 @@
       <c r="L280" t="s">
         <v>917</v>
       </c>
+      <c r="M280" t="s">
+        <v>69</v>
+      </c>
     </row>
     <row r="281" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B281" s="3" t="s">
@@ -12437,6 +12452,9 @@
       <c r="K281" t="s">
         <v>667</v>
       </c>
+      <c r="M281" t="s">
+        <v>69</v>
+      </c>
     </row>
     <row r="282" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B282" s="3" t="s">
@@ -12459,6 +12477,9 @@
       <c r="K282" t="s">
         <v>668</v>
       </c>
+      <c r="M282" t="s">
+        <v>69</v>
+      </c>
     </row>
     <row r="283" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B283" s="3" t="s">
@@ -12481,6 +12502,9 @@
       <c r="K283" t="s">
         <v>668</v>
       </c>
+      <c r="M283" t="s">
+        <v>69</v>
+      </c>
     </row>
     <row r="284" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B284" s="3" t="s">
@@ -12493,7 +12517,7 @@
         <v>61</v>
       </c>
       <c r="E284" t="s">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="F284" t="s">
         <v>431</v>
@@ -12503,6 +12527,9 @@
       <c r="K284" t="s">
         <v>669</v>
       </c>
+      <c r="M284" t="s">
+        <v>69</v>
+      </c>
     </row>
     <row r="285" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B285" s="3" t="s">
@@ -12515,7 +12542,7 @@
         <v>61</v>
       </c>
       <c r="E285" t="s">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="F285" t="s">
         <v>427</v>
@@ -12532,6 +12559,9 @@
       </c>
       <c r="L285" t="s">
         <v>918</v>
+      </c>
+      <c r="M285" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="286" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
@@ -12555,6 +12585,9 @@
       <c r="L286" t="s">
         <v>919</v>
       </c>
+      <c r="M286" t="s">
+        <v>69</v>
+      </c>
     </row>
     <row r="287" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B287" s="3" t="s">
@@ -12581,6 +12614,9 @@
       </c>
       <c r="K287" t="s">
         <v>672</v>
+      </c>
+      <c r="M287" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="288" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
@@ -12601,8 +12637,11 @@
       <c r="K288" t="s">
         <v>673</v>
       </c>
-    </row>
-    <row r="289" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="M288" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="289" spans="2:13" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B289" s="3" t="s">
         <v>360</v>
       </c>
@@ -12613,7 +12652,7 @@
         <v>61</v>
       </c>
       <c r="E289" t="s">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="F289" t="s">
         <v>431</v>
@@ -12626,8 +12665,11 @@
       <c r="K289" t="s">
         <v>674</v>
       </c>
-    </row>
-    <row r="290" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="M289" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="290" spans="2:13" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B290" s="3" t="s">
         <v>361</v>
       </c>
@@ -12651,8 +12693,11 @@
       <c r="L290" t="s">
         <v>920</v>
       </c>
-    </row>
-    <row r="291" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="M290" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="291" spans="2:13" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B291" s="3" t="s">
         <v>362</v>
       </c>
@@ -12673,8 +12718,11 @@
       <c r="K291" t="s">
         <v>675</v>
       </c>
-    </row>
-    <row r="292" spans="2:12" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="M291" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="292" spans="2:13" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B292" s="3" t="s">
         <v>363</v>
       </c>
@@ -12701,8 +12749,11 @@
       <c r="L292" t="s">
         <v>921</v>
       </c>
-    </row>
-    <row r="293" spans="2:12" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="M292" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="293" spans="2:13" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B293" s="3" t="s">
         <v>364</v>
       </c>
@@ -12723,8 +12774,11 @@
       <c r="K293" t="s">
         <v>677</v>
       </c>
-    </row>
-    <row r="294" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="M293" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="294" spans="2:13" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B294" s="3" t="s">
         <v>365</v>
       </c>
@@ -12748,8 +12802,11 @@
       <c r="L294" t="s">
         <v>922</v>
       </c>
-    </row>
-    <row r="295" spans="2:12" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="M294" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="295" spans="2:13" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B295" s="3" t="s">
         <v>366</v>
       </c>
@@ -12773,8 +12830,11 @@
       <c r="L295" t="s">
         <v>923</v>
       </c>
-    </row>
-    <row r="296" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="M295" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="296" spans="2:13" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B296" s="3" t="s">
         <v>367</v>
       </c>
@@ -12798,8 +12858,11 @@
       <c r="K296" t="s">
         <v>679</v>
       </c>
-    </row>
-    <row r="297" spans="2:12" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="M296" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="297" spans="2:13" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B297" s="3" t="s">
         <v>368</v>
       </c>
@@ -12810,7 +12873,7 @@
         <v>61</v>
       </c>
       <c r="E297" t="s">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="F297" t="s">
         <v>431</v>
@@ -12823,8 +12886,11 @@
       <c r="K297" t="s">
         <v>680</v>
       </c>
-    </row>
-    <row r="298" spans="2:12" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="M297" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="298" spans="2:13" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B298" s="3" t="s">
         <v>369</v>
       </c>
@@ -12835,7 +12901,7 @@
         <v>61</v>
       </c>
       <c r="E298" t="s">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="F298" t="s">
         <v>427</v>
@@ -12850,8 +12916,11 @@
       <c r="K298" t="s">
         <v>681</v>
       </c>
-    </row>
-    <row r="299" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="M298" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="299" spans="2:13" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B299" s="3" t="s">
         <v>370</v>
       </c>
@@ -12862,7 +12931,7 @@
         <v>866</v>
       </c>
       <c r="E299" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="F299" t="s">
         <v>431</v>
@@ -12872,8 +12941,11 @@
       <c r="K299" t="s">
         <v>682</v>
       </c>
-    </row>
-    <row r="300" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="M299" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="300" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B300" s="3" t="s">
         <v>371</v>
       </c>
@@ -12884,7 +12956,7 @@
         <v>61</v>
       </c>
       <c r="E300" t="s">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="F300" t="s">
         <v>431</v>
@@ -12897,8 +12969,11 @@
       <c r="K300" t="s">
         <v>683</v>
       </c>
-    </row>
-    <row r="301" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="M300" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="301" spans="2:13" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B301" s="3" t="s">
         <v>372</v>
       </c>
@@ -12916,8 +12991,11 @@
       <c r="K301" t="s">
         <v>417</v>
       </c>
-    </row>
-    <row r="302" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="M301" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="302" spans="2:13" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B302" s="3" t="s">
         <v>373</v>
       </c>
@@ -12941,8 +13019,11 @@
       <c r="K302" t="s">
         <v>683</v>
       </c>
-    </row>
-    <row r="303" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="M302" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="303" spans="2:13" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B303" s="3" t="s">
         <v>374</v>
       </c>
@@ -12960,8 +13041,11 @@
       <c r="K303" t="s">
         <v>684</v>
       </c>
-    </row>
-    <row r="304" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="M303" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="304" spans="2:13" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B304" s="3" t="s">
         <v>375</v>
       </c>
@@ -12982,8 +13066,11 @@
       <c r="K304" t="s">
         <v>685</v>
       </c>
-    </row>
-    <row r="305" spans="2:12" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="M304" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="305" spans="2:13" ht="57.6" x14ac:dyDescent="0.3">
       <c r="B305" s="3" t="s">
         <v>376</v>
       </c>
@@ -12994,7 +13081,7 @@
         <v>61</v>
       </c>
       <c r="E305" t="s">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="F305" t="s">
         <v>427</v>
@@ -13004,8 +13091,11 @@
       <c r="K305" t="s">
         <v>686</v>
       </c>
-    </row>
-    <row r="306" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="M305" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="306" spans="2:13" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B306" s="3" t="s">
         <v>377</v>
       </c>
@@ -13029,8 +13119,11 @@
       <c r="K306" t="s">
         <v>683</v>
       </c>
-    </row>
-    <row r="307" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="M306" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="307" spans="2:13" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B307" s="3" t="s">
         <v>378</v>
       </c>
@@ -13051,8 +13144,11 @@
       <c r="K307" t="s">
         <v>687</v>
       </c>
-    </row>
-    <row r="308" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="M307" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="308" spans="2:13" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B308" s="3" t="s">
         <v>379</v>
       </c>
@@ -13070,8 +13166,11 @@
       <c r="K308" t="s">
         <v>688</v>
       </c>
-    </row>
-    <row r="309" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="M308" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="309" spans="2:13" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B309" s="3" t="s">
         <v>380</v>
       </c>
@@ -13092,8 +13191,11 @@
       <c r="K309" t="s">
         <v>688</v>
       </c>
-    </row>
-    <row r="310" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="M309" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="310" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B310" s="3" t="s">
         <v>381</v>
       </c>
@@ -13104,7 +13206,7 @@
         <v>61</v>
       </c>
       <c r="E310" t="s">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="F310" t="s">
         <v>431</v>
@@ -13122,8 +13224,11 @@
       <c r="L310" t="s">
         <v>924</v>
       </c>
-    </row>
-    <row r="311" spans="2:12" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="M310" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="311" spans="2:13" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B311" s="3" t="s">
         <v>382</v>
       </c>
@@ -13144,8 +13249,11 @@
       <c r="K311" t="s">
         <v>688</v>
       </c>
-    </row>
-    <row r="312" spans="2:12" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="M311" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="312" spans="2:13" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B312" s="3" t="s">
         <v>383</v>
       </c>
@@ -13169,8 +13277,11 @@
       <c r="K312" t="s">
         <v>683</v>
       </c>
-    </row>
-    <row r="313" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="M312" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="313" spans="2:13" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B313" s="3" t="s">
         <v>384</v>
       </c>
@@ -13181,7 +13292,7 @@
         <v>61</v>
       </c>
       <c r="E313" t="s">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="F313" t="s">
         <v>431</v>
@@ -13191,8 +13302,11 @@
       <c r="K313" t="s">
         <v>685</v>
       </c>
-    </row>
-    <row r="314" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="M313" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="314" spans="2:13" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B314" s="3" t="s">
         <v>385</v>
       </c>
@@ -13203,7 +13317,7 @@
         <v>61</v>
       </c>
       <c r="E314" t="s">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="F314" t="s">
         <v>431</v>
@@ -13216,8 +13330,11 @@
       <c r="K314" t="s">
         <v>689</v>
       </c>
-    </row>
-    <row r="315" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="M314" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="315" spans="2:13" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B315" s="3" t="s">
         <v>386</v>
       </c>
@@ -13238,8 +13355,11 @@
       <c r="K315" t="s">
         <v>688</v>
       </c>
-    </row>
-    <row r="316" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="M315" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="316" spans="2:13" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B316" s="3" t="s">
         <v>387</v>
       </c>
@@ -13263,8 +13383,11 @@
       <c r="K316" t="s">
         <v>690</v>
       </c>
-    </row>
-    <row r="317" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="M316" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="317" spans="2:13" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B317" s="3" t="s">
         <v>388</v>
       </c>
@@ -13288,8 +13411,11 @@
       <c r="K317" t="s">
         <v>690</v>
       </c>
-    </row>
-    <row r="318" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="M317" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="318" spans="2:13" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B318" s="3" t="s">
         <v>389</v>
       </c>
@@ -13313,8 +13439,11 @@
       <c r="L318" t="s">
         <v>925</v>
       </c>
-    </row>
-    <row r="319" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="M318" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="319" spans="2:13" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B319" s="3" t="s">
         <v>390</v>
       </c>
@@ -13332,8 +13461,11 @@
       <c r="K319" t="s">
         <v>688</v>
       </c>
-    </row>
-    <row r="320" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="M319" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="320" spans="2:13" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B320" s="3" t="s">
         <v>391</v>
       </c>
@@ -13357,8 +13489,11 @@
       <c r="L320" t="s">
         <v>926</v>
       </c>
-    </row>
-    <row r="321" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="M320" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="321" spans="2:13" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B321" s="3" t="s">
         <v>392</v>
       </c>
@@ -13384,8 +13519,11 @@
       <c r="K321" t="s">
         <v>683</v>
       </c>
-    </row>
-    <row r="322" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="M321" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="322" spans="2:13" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B322" s="3" t="s">
         <v>393</v>
       </c>
@@ -13396,7 +13534,7 @@
         <v>62</v>
       </c>
       <c r="E322" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="F322" t="s">
         <v>431</v>
@@ -13412,8 +13550,11 @@
       <c r="L322" t="s">
         <v>927</v>
       </c>
-    </row>
-    <row r="323" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="M322" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="323" spans="2:13" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B323" s="3" t="s">
         <v>394</v>
       </c>
@@ -13434,8 +13575,11 @@
       <c r="K323" t="s">
         <v>688</v>
       </c>
-    </row>
-    <row r="324" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="M323" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="324" spans="2:13" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B324" s="3" t="s">
         <v>395</v>
       </c>
@@ -13453,8 +13597,11 @@
       <c r="K324" t="s">
         <v>417</v>
       </c>
-    </row>
-    <row r="325" spans="2:12" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="M324" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="325" spans="2:13" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B325" s="3" t="s">
         <v>396</v>
       </c>
@@ -13478,8 +13625,11 @@
       <c r="L325" t="s">
         <v>928</v>
       </c>
-    </row>
-    <row r="326" spans="2:12" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="M325" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="326" spans="2:13" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B326" s="3" t="s">
         <v>397</v>
       </c>
@@ -13503,8 +13653,11 @@
       <c r="L326" t="s">
         <v>929</v>
       </c>
-    </row>
-    <row r="327" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="M326" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="327" spans="2:13" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B327" s="3" t="s">
         <v>398</v>
       </c>
@@ -13522,8 +13675,11 @@
       <c r="K327" t="s">
         <v>692</v>
       </c>
-    </row>
-    <row r="328" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="M327" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="328" spans="2:13" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B328" s="3" t="s">
         <v>399</v>
       </c>
@@ -13534,7 +13690,7 @@
         <v>61</v>
       </c>
       <c r="E328" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="F328" t="s">
         <v>431</v>
@@ -13544,8 +13700,11 @@
       <c r="K328" t="s">
         <v>419</v>
       </c>
-    </row>
-    <row r="329" spans="2:12" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="M328" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="329" spans="2:13" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B329" s="3" t="s">
         <v>400</v>
       </c>
@@ -13566,8 +13725,11 @@
       <c r="K329" t="s">
         <v>692</v>
       </c>
-    </row>
-    <row r="330" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="M329" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="330" spans="2:13" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B330" s="3" t="s">
         <v>401</v>
       </c>
@@ -13591,8 +13753,11 @@
       <c r="L330" t="s">
         <v>930</v>
       </c>
-    </row>
-    <row r="331" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="M330" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="331" spans="2:13" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B331" s="3" t="s">
         <v>402</v>
       </c>
@@ -13616,8 +13781,11 @@
       <c r="L331" t="s">
         <v>931</v>
       </c>
-    </row>
-    <row r="332" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="M331" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="332" spans="2:13" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B332" s="3" t="s">
         <v>403</v>
       </c>
@@ -13638,8 +13806,11 @@
       <c r="K332" t="s">
         <v>695</v>
       </c>
-    </row>
-    <row r="333" spans="2:12" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="M332" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="333" spans="2:13" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B333" s="3" t="s">
         <v>404</v>
       </c>
@@ -13660,8 +13831,11 @@
       <c r="K333" t="s">
         <v>696</v>
       </c>
-    </row>
-    <row r="334" spans="2:12" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="M333" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="334" spans="2:13" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B334" s="3" t="s">
         <v>405</v>
       </c>
@@ -13682,8 +13856,11 @@
       <c r="K334" t="s">
         <v>696</v>
       </c>
-    </row>
-    <row r="335" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="M334" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="335" spans="2:13" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B335" s="3" t="s">
         <v>406</v>
       </c>
@@ -13704,8 +13881,11 @@
       <c r="K335" t="s">
         <v>696</v>
       </c>
-    </row>
-    <row r="336" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="M335" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="336" spans="2:13" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B336" s="3" t="s">
         <v>407</v>
       </c>
@@ -13726,6 +13906,9 @@
       <c r="K336" t="s">
         <v>696</v>
       </c>
+      <c r="M336" t="s">
+        <v>69</v>
+      </c>
     </row>
     <row r="337" spans="2:13" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B337" s="3" t="s">
@@ -13738,7 +13921,7 @@
         <v>61</v>
       </c>
       <c r="E337" t="s">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="F337" t="s">
         <v>431</v>
@@ -13752,6 +13935,9 @@
       </c>
       <c r="K337" t="s">
         <v>697</v>
+      </c>
+      <c r="M337" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="338" spans="2:13" ht="28.8" x14ac:dyDescent="0.3">
@@ -13775,6 +13961,9 @@
       <c r="K338" t="s">
         <v>698</v>
       </c>
+      <c r="M338" t="s">
+        <v>69</v>
+      </c>
     </row>
     <row r="339" spans="2:13" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B339" s="3" t="s">
@@ -13800,6 +13989,9 @@
       <c r="K339" t="s">
         <v>699</v>
       </c>
+      <c r="M339" t="s">
+        <v>69</v>
+      </c>
     </row>
     <row r="340" spans="2:13" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B340" s="3" t="s">
@@ -13819,6 +14011,9 @@
       <c r="K340" t="s">
         <v>420</v>
       </c>
+      <c r="M340" t="s">
+        <v>69</v>
+      </c>
     </row>
     <row r="341" spans="2:13" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B341" s="3" t="s">
@@ -13841,6 +14036,9 @@
       <c r="L341" t="s">
         <v>932</v>
       </c>
+      <c r="M341" t="s">
+        <v>69</v>
+      </c>
     </row>
     <row r="342" spans="2:13" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B342" s="3" t="s">
@@ -13869,6 +14067,9 @@
       <c r="L342" t="s">
         <v>933</v>
       </c>
+      <c r="M342" t="s">
+        <v>69</v>
+      </c>
     </row>
     <row r="343" spans="2:13" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B343" s="3" t="s">
@@ -14006,6 +14207,9 @@
       <c r="L348" t="s">
         <v>934</v>
       </c>
+      <c r="M348" t="s">
+        <v>69</v>
+      </c>
     </row>
     <row r="349" spans="2:13" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B349" s="3" t="s">
@@ -14028,6 +14232,9 @@
       <c r="L349" t="s">
         <v>935</v>
       </c>
+      <c r="M349" t="s">
+        <v>69</v>
+      </c>
     </row>
     <row r="350" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B350" s="3" t="s">
@@ -16326,7 +16533,7 @@
         <v>873</v>
       </c>
       <c r="E445" t="s">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="F445" t="s">
         <v>428</v>
@@ -19500,15 +19707,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100959716F11FB6F9409089B98D1C11D330" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="bc55ac45923017d94ee4534da3224188">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="2e20d828-e3fd-41fd-921c-fbe0ff523ae8" xmlns:ns3="adfc7943-f9ee-4478-a01e-ebfcb6e54f53" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="5bc17ad4f23ab8382a0bb5b03decca58" ns2:_="" ns3:_="">
     <xsd:import namespace="2e20d828-e3fd-41fd-921c-fbe0ff523ae8"/>
@@ -19763,6 +19961,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -19775,14 +19982,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{737DCCA1-99B2-40A5-A4E9-9FBBAC380C60}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5CE6A3B7-F954-4629-B802-2205DECE6851}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -19801,6 +20000,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{737DCCA1-99B2-40A5-A4E9-9FBBAC380C60}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{407A8743-A532-48E3-9004-715BF423F4DA}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
Add 33 Eye-Q AI_CORE + beta integration tasks (#490-#522): ABI.Unity issues #1047-#1079
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/project_time_sheet.xlsx
+++ b/project_time_sheet.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30228"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B052D40-1573-4692-A87F-0EE66AEB1929}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03C006B5-D551-4B1A-A191-E0B596FEA2B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2723" uniqueCount="982">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2954" uniqueCount="1082">
   <si>
     <t xml:space="preserve">  Project Time Sheet — User Guide</t>
   </si>
@@ -2983,6 +2983,306 @@
   </si>
   <si>
     <t>Implemented and committed as b2ea7dc; iPadOS does not permit PWA to hide system indicators automatically</t>
+  </si>
+  <si>
+    <t>Integrate AI_CORE inside EyeQ settings</t>
+  </si>
+  <si>
+    <t>Add authenticated AI_CORE page under Settings with embedded AI Core UI.</t>
+  </si>
+  <si>
+    <t>Iframe embedding and authenticated access implemented.</t>
+  </si>
+  <si>
+    <t>Make AI_CORE iframe responsive</t>
+  </si>
+  <si>
+    <t>Use explicit embedded URL, automatic port handling, full-screen behavior, Web Browser compatibility, light-mode support, and remove open-in-new-tab control.</t>
+  </si>
+  <si>
+    <t>Desktop and WEB Browser layout adjustments applied.</t>
+  </si>
+  <si>
+    <t>Add AI_CORE submenu to EyeQ</t>
+  </si>
+  <si>
+    <t>Expose AI_CORE workflow sections as EyeQ Settings submenu items and hide them when the feature is disabled.</t>
+  </si>
+  <si>
+    <t>Controlled by the AICoreAccess general setting.</t>
+  </si>
+  <si>
+    <t>Protect AI_CORE pages with authentication</t>
+  </si>
+  <si>
+    <t>Prevent logged-out users from opening AI_CORE URLs directly.</t>
+  </si>
+  <si>
+    <t>Direct URL access now follows EyeQ authentication.</t>
+  </si>
+  <si>
+    <t>Enable EyeQ remote access</t>
+  </si>
+  <si>
+    <t>Make EyeQ and AI_CORE reachable from a tablet on the plant network and diagnose access failures.</t>
+  </si>
+  <si>
+    <t>Binding/access troubleshooting completed; device/network firewall validation may still be required.</t>
+  </si>
+  <si>
+    <t>Define EyeQ to AI_CORE communication</t>
+  </si>
+  <si>
+    <t>Document and implement communication responsibilities, API usage, and result delivery between both applications.</t>
+  </si>
+  <si>
+    <t>Frame-correlated trigger/result architecture selected.</t>
+  </si>
+  <si>
+    <t>Implement EyeQ Output workflow node</t>
+  </si>
+  <si>
+    <t>Create a configurable AI_CORE node that maps detections and measurements into EyeQ scan data with retries and authentication.</t>
+  </si>
+  <si>
+    <t>Existing node posts authenticated scan payloads.</t>
+  </si>
+  <si>
+    <t>Fix EyeQ results not appearing</t>
+  </si>
+  <si>
+    <t>Diagnose and correct the path from AI_CORE output to EyeQ measurements, database records, and dashboards.</t>
+  </si>
+  <si>
+    <t>Ingest and dashboard scan-source handling corrected.</t>
+  </si>
+  <si>
+    <t>Fix Planar World Metrology reference handling</t>
+  </si>
+  <si>
+    <t>Resolve empty planar references and add full-image fallback when a connected reference image exists.</t>
+  </si>
+  <si>
+    <t>Clear validation message and fallback test added.</t>
+  </si>
+  <si>
+    <t>Support rectangle and four-corner planar selection</t>
+  </si>
+  <si>
+    <t>Allow Planar World Metrology to use either a rectangular crop or four manually selected corners.</t>
+  </si>
+  <si>
+    <t>UI mode selector and persistence implemented.</t>
+  </si>
+  <si>
+    <t>Design photoeye-triggered inspection workflow</t>
+  </si>
+  <si>
+    <t>Evaluate options for EyeQ photoeye trigger, AI_CORE frame capture, workflow processing, and result return.</t>
+  </si>
+  <si>
+    <t>Option 1 selected: synchronous short wait plus asynchronous fallback.</t>
+  </si>
+  <si>
+    <t>Implement photoeye inspection trigger API</t>
+  </si>
+  <si>
+    <t>EyeQ sends frameId/triggerId to AI_CORE, AI_CORE runs the active workflow, and returns a completed response or 202 job.</t>
+  </si>
+  <si>
+    <t>Endpoints implemented: /api/inspection/trigger and job status route.</t>
+  </si>
+  <si>
+    <t>Implement scan-result ingest with base64 images</t>
+  </si>
+  <si>
+    <t>Add EyeQ endpoint to receive scan data, original image, processed image, and correlated frame identifiers.</t>
+  </si>
+  <si>
+    <t>Images are stored under EyeQ inference image storage.</t>
+  </si>
+  <si>
+    <t>Restart and validate both applications</t>
+  </si>
+  <si>
+    <t>Rebuild/publish EyeQ, restart EyeQ and AI_CORE, and verify ports and service health after changes.</t>
+  </si>
+  <si>
+    <t>EyeQ port 5000 and AI_CORE port 8000 verified.</t>
+  </si>
+  <si>
+    <t>Compare beta with dev/md-ui</t>
+  </si>
+  <si>
+    <t>Identify merge constraints, conflicts, and overlapping changes before integration.</t>
+  </si>
+  <si>
+    <t>Eight content conflicts identified.</t>
+  </si>
+  <si>
+    <t>Create integration branch</t>
+  </si>
+  <si>
+    <t>Create dev/md-ui-beta-integration from dev/md-ui for safe beta integration.</t>
+  </si>
+  <si>
+    <t>Isolated branch used; beta and dev branches preserved.</t>
+  </si>
+  <si>
+    <t>Integrate beta backend and configuration</t>
+  </si>
+  <si>
+    <t>Merge beta model library, deployment, training, inspection, and runtime changes.</t>
+  </si>
+  <si>
+    <t>Preserved dev camera, Agent, synthetic-data, and multi-camera settings.</t>
+  </si>
+  <si>
+    <t>Integrate beta frontend</t>
+  </si>
+  <si>
+    <t>Merge model library, deployment, training, workflow, Agent, PWA, and iframe UI changes.</t>
+  </si>
+  <si>
+    <t>Resolved conflicts in index.html, training UI, and workflow UI.</t>
+  </si>
+  <si>
+    <t>Preserve multi-camera and camera networking</t>
+  </si>
+  <si>
+    <t>Keep jumbo-frame settings, camera serial configuration, stitching, crop, caching, and calibration behavior from dev.</t>
+  </si>
+  <si>
+    <t>Dev camera/network settings were intentionally retained.</t>
+  </si>
+  <si>
+    <t>Preserve serial-aware calibration</t>
+  </si>
+  <si>
+    <t>Keep serial-aware calibration and integrate beta calibration-related changes.</t>
+  </si>
+  <si>
+    <t>Calibration routes and profiles remain available.</t>
+  </si>
+  <si>
+    <t>Integrate workflow deployment support</t>
+  </si>
+  <si>
+    <t>Add beta's workflow deployment, runtime history, start/stop, and rollback functionality.</t>
+  </si>
+  <si>
+    <t>Deployment API and UI are available.</t>
+  </si>
+  <si>
+    <t>Integrate model library and training features</t>
+  </si>
+  <si>
+    <t>Add model import, benchmark, deployment, batch workspace, autolabel, review, and publish features.</t>
+  </si>
+  <si>
+    <t>Model and training endpoints respond successfully.</t>
+  </si>
+  <si>
+    <t>Reintroduce synthetic-data support</t>
+  </si>
+  <si>
+    <t>Preserve synthetic-data generation, metadata lineage, review, and train-only grouping.</t>
+  </si>
+  <si>
+    <t>Synthetic data remains experimental and available in Training.</t>
+  </si>
+  <si>
+    <t>Fix dataset merge compatibility</t>
+  </si>
+  <si>
+    <t>Preserve beta batch metadata while maintaining dev synthetic metadata and legacy positional API compatibility.</t>
+  </si>
+  <si>
+    <t>Dataset tests pass.</t>
+  </si>
+  <si>
+    <t>Fix detector test instability</t>
+  </si>
+  <si>
+    <t>Make OpenCV k-means deterministic by resetting its process-global RNG seed.</t>
+  </si>
+  <si>
+    <t>Removed order-dependent test failure.</t>
+  </si>
+  <si>
+    <t>Update documentation coverage</t>
+  </si>
+  <si>
+    <t>Add the beta workflow node documentation, including Misshapen Geometry Check.</t>
+  </si>
+  <si>
+    <t>Documentation validation passes.</t>
+  </si>
+  <si>
+    <t>Run automated validation</t>
+  </si>
+  <si>
+    <t>Execute syntax checks and the complete automated test suite.</t>
+  </si>
+  <si>
+    <t>677 tests passed.</t>
+  </si>
+  <si>
+    <t>Restart and smoke-test the application</t>
+  </si>
+  <si>
+    <t>Restart the service and verify key pages and APIs.</t>
+  </si>
+  <si>
+    <t>Workflow, training, models, Agent, synthetic data, deployment, and camera APIs responded.</t>
+  </si>
+  <si>
+    <t>Live-test both Ace cameras</t>
+  </si>
+  <si>
+    <t>Verify both physical Ace cameras after merge.</t>
+  </si>
+  <si>
+    <t>On Hold</t>
+  </si>
+  <si>
+    <t>No Pylon devices were discoverable on the host during testing. Requires cameras/network connection.</t>
+  </si>
+  <si>
+    <t>Compare integration branch with beta</t>
+  </si>
+  <si>
+    <t>Confirm whether dev/md-ui-beta-integration can be deleted safely.</t>
+  </si>
+  <si>
+    <t>Beta contains the integration commit and no integration-only changes remain.</t>
+  </si>
+  <si>
+    <t>Embed AI Core inside the EyeQ user interface</t>
+  </si>
+  <si>
+    <t>Created the authenticated /settings/ai_core EyeQ page, embedded the AI Core application in an iframe, generated its URL from EyeQ configuration.</t>
+  </si>
+  <si>
+    <t>Git commit 6a6b7d1a.</t>
+  </si>
+  <si>
+    <t>Add tablet-responsive support for the EyeQ AI Core view</t>
+  </si>
+  <si>
+    <t>Updated EyeQ application-level viewport/scaling behavior and refined the AI Core page so the embedded interface works more reliably on tablet-sized displays.</t>
+  </si>
+  <si>
+    <t>Git commit 04d09734.</t>
+  </si>
+  <si>
+    <t>Control AI Core visibility and access from EyeQ settings</t>
+  </si>
+  <si>
+    <t>Added an AI Core feature setting and notification flow, exposed an enable/disable switch in General Settings, dynamically showed or hid the AI Core menu.</t>
+  </si>
+  <si>
+    <t>Git commit b699b85f.</t>
   </si>
 </sst>
 </file>
@@ -4864,7 +5164,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:N1020"/>
+  <dimension ref="A1:N1053"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="7.6640625" customWidth="1"/>
@@ -19578,6 +19878,1062 @@
         <v>981</v>
       </c>
       <c r="M1020" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1021" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A1021">
+        <v>490</v>
+      </c>
+      <c r="B1021" s="3" t="s">
+        <v>982</v>
+      </c>
+      <c r="C1021" s="3" t="s">
+        <v>983</v>
+      </c>
+      <c r="D1021" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1021" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1021" t="s">
+        <v>431</v>
+      </c>
+      <c r="H1021">
+        <v>4</v>
+      </c>
+      <c r="J1021" s="42">
+        <v>46252</v>
+      </c>
+      <c r="L1021" t="s">
+        <v>984</v>
+      </c>
+      <c r="M1021" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1022" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1022">
+        <v>491</v>
+      </c>
+      <c r="B1022" s="3" t="s">
+        <v>985</v>
+      </c>
+      <c r="C1022" s="3" t="s">
+        <v>986</v>
+      </c>
+      <c r="D1022" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1022" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1022" t="s">
+        <v>431</v>
+      </c>
+      <c r="H1022">
+        <v>5</v>
+      </c>
+      <c r="J1022" s="42">
+        <v>46252</v>
+      </c>
+      <c r="L1022" t="s">
+        <v>987</v>
+      </c>
+      <c r="M1022" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1023" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1023">
+        <v>492</v>
+      </c>
+      <c r="B1023" s="3" t="s">
+        <v>988</v>
+      </c>
+      <c r="C1023" s="3" t="s">
+        <v>989</v>
+      </c>
+      <c r="D1023" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1023" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1023" t="s">
+        <v>431</v>
+      </c>
+      <c r="H1023">
+        <v>3</v>
+      </c>
+      <c r="J1023" s="42">
+        <v>46252</v>
+      </c>
+      <c r="L1023" t="s">
+        <v>990</v>
+      </c>
+      <c r="M1023" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1024" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A1024">
+        <v>493</v>
+      </c>
+      <c r="B1024" s="3" t="s">
+        <v>991</v>
+      </c>
+      <c r="C1024" s="3" t="s">
+        <v>992</v>
+      </c>
+      <c r="D1024" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1024" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1024" t="s">
+        <v>427</v>
+      </c>
+      <c r="H1024">
+        <v>3</v>
+      </c>
+      <c r="J1024" s="42">
+        <v>46252</v>
+      </c>
+      <c r="L1024" t="s">
+        <v>993</v>
+      </c>
+      <c r="M1024" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1025" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1025">
+        <v>494</v>
+      </c>
+      <c r="B1025" s="3" t="s">
+        <v>994</v>
+      </c>
+      <c r="C1025" s="3" t="s">
+        <v>995</v>
+      </c>
+      <c r="D1025" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1025" t="s">
+        <v>73</v>
+      </c>
+      <c r="F1025" t="s">
+        <v>427</v>
+      </c>
+      <c r="H1025">
+        <v>3</v>
+      </c>
+      <c r="J1025" s="42">
+        <v>46252</v>
+      </c>
+      <c r="L1025" t="s">
+        <v>996</v>
+      </c>
+      <c r="M1025" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1026" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1026">
+        <v>495</v>
+      </c>
+      <c r="B1026" s="3" t="s">
+        <v>997</v>
+      </c>
+      <c r="C1026" s="3" t="s">
+        <v>998</v>
+      </c>
+      <c r="D1026" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1026" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1026" t="s">
+        <v>427</v>
+      </c>
+      <c r="H1026">
+        <v>4</v>
+      </c>
+      <c r="J1026" s="42">
+        <v>46252</v>
+      </c>
+      <c r="L1026" t="s">
+        <v>999</v>
+      </c>
+      <c r="M1026" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1027" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1027">
+        <v>496</v>
+      </c>
+      <c r="B1027" s="3" t="s">
+        <v>1000</v>
+      </c>
+      <c r="C1027" s="3" t="s">
+        <v>1001</v>
+      </c>
+      <c r="D1027" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1027" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1027" t="s">
+        <v>427</v>
+      </c>
+      <c r="H1027">
+        <v>8</v>
+      </c>
+      <c r="J1027" s="42">
+        <v>46252</v>
+      </c>
+      <c r="L1027" t="s">
+        <v>1002</v>
+      </c>
+      <c r="M1027" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1028" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1028">
+        <v>497</v>
+      </c>
+      <c r="B1028" s="3" t="s">
+        <v>1003</v>
+      </c>
+      <c r="C1028" s="3" t="s">
+        <v>1004</v>
+      </c>
+      <c r="D1028" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1028" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1028" t="s">
+        <v>427</v>
+      </c>
+      <c r="H1028">
+        <v>6</v>
+      </c>
+      <c r="J1028" s="42">
+        <v>46252</v>
+      </c>
+      <c r="L1028" t="s">
+        <v>1005</v>
+      </c>
+      <c r="M1028" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1029" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1029">
+        <v>498</v>
+      </c>
+      <c r="B1029" s="3" t="s">
+        <v>1006</v>
+      </c>
+      <c r="C1029" s="3" t="s">
+        <v>1007</v>
+      </c>
+      <c r="D1029" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1029" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1029" t="s">
+        <v>427</v>
+      </c>
+      <c r="H1029">
+        <v>6</v>
+      </c>
+      <c r="J1029" s="42">
+        <v>46252</v>
+      </c>
+      <c r="L1029" t="s">
+        <v>1008</v>
+      </c>
+      <c r="M1029" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1030" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1030">
+        <v>499</v>
+      </c>
+      <c r="B1030" s="3" t="s">
+        <v>1009</v>
+      </c>
+      <c r="C1030" s="3" t="s">
+        <v>1010</v>
+      </c>
+      <c r="D1030" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1030" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1030" t="s">
+        <v>427</v>
+      </c>
+      <c r="H1030">
+        <v>5</v>
+      </c>
+      <c r="J1030" s="42">
+        <v>46252</v>
+      </c>
+      <c r="L1030" t="s">
+        <v>1011</v>
+      </c>
+      <c r="M1030" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1031" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1031">
+        <v>500</v>
+      </c>
+      <c r="B1031" s="3" t="s">
+        <v>1012</v>
+      </c>
+      <c r="C1031" s="3" t="s">
+        <v>1013</v>
+      </c>
+      <c r="D1031" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1031" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1031" t="s">
+        <v>427</v>
+      </c>
+      <c r="H1031">
+        <v>4</v>
+      </c>
+      <c r="J1031" s="42">
+        <v>46252</v>
+      </c>
+      <c r="L1031" t="s">
+        <v>1014</v>
+      </c>
+      <c r="M1031" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1032" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1032">
+        <v>501</v>
+      </c>
+      <c r="B1032" s="3" t="s">
+        <v>1015</v>
+      </c>
+      <c r="C1032" s="3" t="s">
+        <v>1016</v>
+      </c>
+      <c r="D1032" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1032" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1032" t="s">
+        <v>427</v>
+      </c>
+      <c r="H1032">
+        <v>12</v>
+      </c>
+      <c r="J1032" s="42">
+        <v>46252</v>
+      </c>
+      <c r="L1032" t="s">
+        <v>1017</v>
+      </c>
+      <c r="M1032" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1033" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1033">
+        <v>502</v>
+      </c>
+      <c r="B1033" s="3" t="s">
+        <v>1018</v>
+      </c>
+      <c r="C1033" s="3" t="s">
+        <v>1019</v>
+      </c>
+      <c r="D1033" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1033" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1033" t="s">
+        <v>427</v>
+      </c>
+      <c r="H1033">
+        <v>8</v>
+      </c>
+      <c r="J1033" s="42">
+        <v>46252</v>
+      </c>
+      <c r="L1033" t="s">
+        <v>1020</v>
+      </c>
+      <c r="M1033" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1034" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1034">
+        <v>503</v>
+      </c>
+      <c r="B1034" s="3" t="s">
+        <v>1021</v>
+      </c>
+      <c r="C1034" s="3" t="s">
+        <v>1022</v>
+      </c>
+      <c r="D1034" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1034" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1034" t="s">
+        <v>427</v>
+      </c>
+      <c r="H1034">
+        <v>3</v>
+      </c>
+      <c r="J1034" s="42">
+        <v>46252</v>
+      </c>
+      <c r="L1034" t="s">
+        <v>1023</v>
+      </c>
+      <c r="M1034" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1035" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A1035">
+        <v>504</v>
+      </c>
+      <c r="B1035" s="3" t="s">
+        <v>1024</v>
+      </c>
+      <c r="C1035" s="3" t="s">
+        <v>1025</v>
+      </c>
+      <c r="D1035" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1035" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1035" t="s">
+        <v>427</v>
+      </c>
+      <c r="H1035">
+        <v>1.5</v>
+      </c>
+      <c r="J1035" s="42">
+        <v>46252</v>
+      </c>
+      <c r="L1035" t="s">
+        <v>1026</v>
+      </c>
+      <c r="M1035" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1036" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A1036">
+        <v>505</v>
+      </c>
+      <c r="B1036" s="3" t="s">
+        <v>1027</v>
+      </c>
+      <c r="C1036" s="3" t="s">
+        <v>1028</v>
+      </c>
+      <c r="D1036" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1036" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1036" t="s">
+        <v>427</v>
+      </c>
+      <c r="H1036">
+        <v>0.5</v>
+      </c>
+      <c r="J1036" s="42">
+        <v>46252</v>
+      </c>
+      <c r="L1036" t="s">
+        <v>1029</v>
+      </c>
+      <c r="M1036" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1037" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A1037">
+        <v>506</v>
+      </c>
+      <c r="B1037" s="3" t="s">
+        <v>1030</v>
+      </c>
+      <c r="C1037" s="3" t="s">
+        <v>1031</v>
+      </c>
+      <c r="D1037" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1037" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1037" t="s">
+        <v>427</v>
+      </c>
+      <c r="H1037">
+        <v>4</v>
+      </c>
+      <c r="J1037" s="42">
+        <v>46252</v>
+      </c>
+      <c r="L1037" t="s">
+        <v>1032</v>
+      </c>
+      <c r="M1037" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1038" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1038">
+        <v>507</v>
+      </c>
+      <c r="B1038" s="3" t="s">
+        <v>1033</v>
+      </c>
+      <c r="C1038" s="3" t="s">
+        <v>1034</v>
+      </c>
+      <c r="D1038" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1038" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1038" t="s">
+        <v>427</v>
+      </c>
+      <c r="H1038">
+        <v>5</v>
+      </c>
+      <c r="J1038" s="42">
+        <v>46252</v>
+      </c>
+      <c r="L1038" t="s">
+        <v>1035</v>
+      </c>
+      <c r="M1038" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1039" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1039">
+        <v>508</v>
+      </c>
+      <c r="B1039" s="3" t="s">
+        <v>1036</v>
+      </c>
+      <c r="C1039" s="3" t="s">
+        <v>1037</v>
+      </c>
+      <c r="D1039" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1039" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1039" t="s">
+        <v>427</v>
+      </c>
+      <c r="H1039">
+        <v>2</v>
+      </c>
+      <c r="J1039" s="42">
+        <v>46252</v>
+      </c>
+      <c r="L1039" t="s">
+        <v>1038</v>
+      </c>
+      <c r="M1039" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1040" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A1040">
+        <v>509</v>
+      </c>
+      <c r="B1040" s="3" t="s">
+        <v>1039</v>
+      </c>
+      <c r="C1040" s="3" t="s">
+        <v>1040</v>
+      </c>
+      <c r="D1040" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1040" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1040" t="s">
+        <v>427</v>
+      </c>
+      <c r="H1040">
+        <v>2</v>
+      </c>
+      <c r="J1040" s="42">
+        <v>46252</v>
+      </c>
+      <c r="L1040" t="s">
+        <v>1041</v>
+      </c>
+      <c r="M1040" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1041" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1041">
+        <v>510</v>
+      </c>
+      <c r="B1041" s="3" t="s">
+        <v>1042</v>
+      </c>
+      <c r="C1041" s="3" t="s">
+        <v>1043</v>
+      </c>
+      <c r="D1041" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1041" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1041" t="s">
+        <v>427</v>
+      </c>
+      <c r="H1041">
+        <v>3</v>
+      </c>
+      <c r="J1041" s="42">
+        <v>46252</v>
+      </c>
+      <c r="L1041" t="s">
+        <v>1044</v>
+      </c>
+      <c r="M1041" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1042" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1042">
+        <v>511</v>
+      </c>
+      <c r="B1042" s="3" t="s">
+        <v>1045</v>
+      </c>
+      <c r="C1042" s="3" t="s">
+        <v>1046</v>
+      </c>
+      <c r="D1042" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1042" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1042" t="s">
+        <v>427</v>
+      </c>
+      <c r="H1042">
+        <v>4</v>
+      </c>
+      <c r="J1042" s="42">
+        <v>46252</v>
+      </c>
+      <c r="L1042" t="s">
+        <v>1047</v>
+      </c>
+      <c r="M1042" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1043" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1043">
+        <v>512</v>
+      </c>
+      <c r="B1043" s="3" t="s">
+        <v>1048</v>
+      </c>
+      <c r="C1043" s="3" t="s">
+        <v>1049</v>
+      </c>
+      <c r="D1043" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1043" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1043" t="s">
+        <v>431</v>
+      </c>
+      <c r="H1043">
+        <v>2</v>
+      </c>
+      <c r="J1043" s="42">
+        <v>46252</v>
+      </c>
+      <c r="L1043" t="s">
+        <v>1050</v>
+      </c>
+      <c r="M1043" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1044" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1044">
+        <v>513</v>
+      </c>
+      <c r="B1044" s="3" t="s">
+        <v>1051</v>
+      </c>
+      <c r="C1044" s="3" t="s">
+        <v>1052</v>
+      </c>
+      <c r="D1044" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1044" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1044" t="s">
+        <v>427</v>
+      </c>
+      <c r="H1044">
+        <v>1.5</v>
+      </c>
+      <c r="J1044" s="42">
+        <v>46252</v>
+      </c>
+      <c r="L1044" t="s">
+        <v>1053</v>
+      </c>
+      <c r="M1044" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1045" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A1045">
+        <v>514</v>
+      </c>
+      <c r="B1045" s="3" t="s">
+        <v>1054</v>
+      </c>
+      <c r="C1045" s="3" t="s">
+        <v>1055</v>
+      </c>
+      <c r="D1045" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1045" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1045" t="s">
+        <v>431</v>
+      </c>
+      <c r="H1045">
+        <v>1</v>
+      </c>
+      <c r="J1045" s="42">
+        <v>46252</v>
+      </c>
+      <c r="L1045" t="s">
+        <v>1056</v>
+      </c>
+      <c r="M1045" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1046" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A1046">
+        <v>515</v>
+      </c>
+      <c r="B1046" s="3" t="s">
+        <v>1057</v>
+      </c>
+      <c r="C1046" s="3" t="s">
+        <v>1058</v>
+      </c>
+      <c r="D1046" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1046" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1046" t="s">
+        <v>431</v>
+      </c>
+      <c r="H1046">
+        <v>1</v>
+      </c>
+      <c r="J1046" s="42">
+        <v>46252</v>
+      </c>
+      <c r="L1046" t="s">
+        <v>1059</v>
+      </c>
+      <c r="M1046" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1047" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A1047">
+        <v>516</v>
+      </c>
+      <c r="B1047" s="3" t="s">
+        <v>1060</v>
+      </c>
+      <c r="C1047" s="3" t="s">
+        <v>1061</v>
+      </c>
+      <c r="D1047" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1047" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1047" t="s">
+        <v>427</v>
+      </c>
+      <c r="H1047">
+        <v>1.5</v>
+      </c>
+      <c r="J1047" s="42">
+        <v>46252</v>
+      </c>
+      <c r="L1047" t="s">
+        <v>1062</v>
+      </c>
+      <c r="M1047" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1048" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A1048">
+        <v>517</v>
+      </c>
+      <c r="B1048" s="3" t="s">
+        <v>1063</v>
+      </c>
+      <c r="C1048" s="3" t="s">
+        <v>1064</v>
+      </c>
+      <c r="D1048" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1048" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1048" t="s">
+        <v>427</v>
+      </c>
+      <c r="H1048">
+        <v>1</v>
+      </c>
+      <c r="J1048" s="42">
+        <v>46252</v>
+      </c>
+      <c r="L1048" t="s">
+        <v>1065</v>
+      </c>
+      <c r="M1048" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1049" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A1049">
+        <v>518</v>
+      </c>
+      <c r="B1049" s="3" t="s">
+        <v>1066</v>
+      </c>
+      <c r="C1049" s="3" t="s">
+        <v>1067</v>
+      </c>
+      <c r="D1049" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1049" t="s">
+        <v>1068</v>
+      </c>
+      <c r="F1049" t="s">
+        <v>427</v>
+      </c>
+      <c r="H1049">
+        <v>2</v>
+      </c>
+      <c r="J1049" s="42">
+        <v>46252</v>
+      </c>
+      <c r="L1049" t="s">
+        <v>1069</v>
+      </c>
+      <c r="M1049" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1050" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A1050">
+        <v>519</v>
+      </c>
+      <c r="B1050" s="3" t="s">
+        <v>1070</v>
+      </c>
+      <c r="C1050" s="3" t="s">
+        <v>1071</v>
+      </c>
+      <c r="D1050" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1050" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1050" t="s">
+        <v>431</v>
+      </c>
+      <c r="H1050">
+        <v>0.5</v>
+      </c>
+      <c r="J1050" s="42">
+        <v>46252</v>
+      </c>
+      <c r="L1050" t="s">
+        <v>1072</v>
+      </c>
+      <c r="M1050" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1051" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1051">
+        <v>520</v>
+      </c>
+      <c r="B1051" s="3" t="s">
+        <v>1073</v>
+      </c>
+      <c r="C1051" s="3" t="s">
+        <v>1074</v>
+      </c>
+      <c r="D1051" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1051" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1051" t="s">
+        <v>427</v>
+      </c>
+      <c r="H1051">
+        <v>2</v>
+      </c>
+      <c r="J1051" s="42">
+        <v>46252</v>
+      </c>
+      <c r="L1051" t="s">
+        <v>1075</v>
+      </c>
+      <c r="M1051" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1052" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1052">
+        <v>521</v>
+      </c>
+      <c r="B1052" s="3" t="s">
+        <v>1076</v>
+      </c>
+      <c r="C1052" s="3" t="s">
+        <v>1077</v>
+      </c>
+      <c r="D1052" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1052" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1052" t="s">
+        <v>427</v>
+      </c>
+      <c r="H1052">
+        <v>1</v>
+      </c>
+      <c r="J1052" s="42">
+        <v>46252</v>
+      </c>
+      <c r="L1052" t="s">
+        <v>1078</v>
+      </c>
+      <c r="M1052" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1053" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1053">
+        <v>522</v>
+      </c>
+      <c r="B1053" s="3" t="s">
+        <v>1079</v>
+      </c>
+      <c r="C1053" s="3" t="s">
+        <v>1080</v>
+      </c>
+      <c r="D1053" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1053" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1053" t="s">
+        <v>427</v>
+      </c>
+      <c r="H1053">
+        <v>2</v>
+      </c>
+      <c r="J1053" s="42">
+        <v>46252</v>
+      </c>
+      <c r="L1053" t="s">
+        <v>1081</v>
+      </c>
+      <c r="M1053" t="s">
         <v>182</v>
       </c>
     </row>
@@ -19707,6 +21063,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100959716F11FB6F9409089B98D1C11D330" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="bc55ac45923017d94ee4534da3224188">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="2e20d828-e3fd-41fd-921c-fbe0ff523ae8" xmlns:ns3="adfc7943-f9ee-4478-a01e-ebfcb6e54f53" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="5bc17ad4f23ab8382a0bb5b03decca58" ns2:_="" ns3:_="">
     <xsd:import namespace="2e20d828-e3fd-41fd-921c-fbe0ff523ae8"/>
@@ -19961,15 +21326,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -19982,6 +21338,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{737DCCA1-99B2-40A5-A4E9-9FBBAC380C60}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5CE6A3B7-F954-4629-B802-2205DECE6851}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -20000,14 +21364,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{737DCCA1-99B2-40A5-A4E9-9FBBAC380C60}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{407A8743-A532-48E3-9004-715BF423F4DA}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
Add 1 Katana IPC task (#523): ABI.Unity issue #1080 - Test IPC last BIOS upgrade with Backoff team
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/project_time_sheet.xlsx
+++ b/project_time_sheet.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30228"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03C006B5-D551-4B1A-A191-E0B596FEA2B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91A1CB4B-2609-4B1E-B10C-A14C0AE29F4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2954" uniqueCount="1082">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2962" uniqueCount="1086">
   <si>
     <t xml:space="preserve">  Project Time Sheet — User Guide</t>
   </si>
@@ -3283,6 +3283,18 @@
   </si>
   <si>
     <t>Git commit b699b85f.</t>
+  </si>
+  <si>
+    <t>Test IPC last BIOS upgrade with Backoff team</t>
+  </si>
+  <si>
+    <t>Test the Beckoff IPC after the last BIOS upgrade with the Backoff team.</t>
+  </si>
+  <si>
+    <t>Issue</t>
+  </si>
+  <si>
+    <t>Beckoff IPC reaches &gt;4 GHz speed; tested with phantom mode and production mode, IPC performs well.</t>
   </si>
 </sst>
 </file>
@@ -5164,7 +5176,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:N1053"/>
+  <dimension ref="A1:N1054"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="7.6640625" customWidth="1"/>
@@ -20935,6 +20947,38 @@
       </c>
       <c r="M1053" t="s">
         <v>182</v>
+      </c>
+    </row>
+    <row r="1054" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A1054">
+        <v>523</v>
+      </c>
+      <c r="B1054" s="3" t="s">
+        <v>1082</v>
+      </c>
+      <c r="C1054" s="3" t="s">
+        <v>1083</v>
+      </c>
+      <c r="D1054" t="s">
+        <v>485</v>
+      </c>
+      <c r="E1054" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1054" t="s">
+        <v>427</v>
+      </c>
+      <c r="H1054">
+        <v>2</v>
+      </c>
+      <c r="K1054" t="s">
+        <v>1084</v>
+      </c>
+      <c r="L1054" t="s">
+        <v>1085</v>
+      </c>
+      <c r="M1054" t="s">
+        <v>69</v>
       </c>
     </row>
   </sheetData>
@@ -21063,15 +21107,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100959716F11FB6F9409089B98D1C11D330" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="bc55ac45923017d94ee4534da3224188">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="2e20d828-e3fd-41fd-921c-fbe0ff523ae8" xmlns:ns3="adfc7943-f9ee-4478-a01e-ebfcb6e54f53" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="5bc17ad4f23ab8382a0bb5b03decca58" ns2:_="" ns3:_="">
     <xsd:import namespace="2e20d828-e3fd-41fd-921c-fbe0ff523ae8"/>
@@ -21326,6 +21361,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -21338,14 +21382,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{737DCCA1-99B2-40A5-A4E9-9FBBAC380C60}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5CE6A3B7-F954-4629-B802-2205DECE6851}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -21364,6 +21400,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{737DCCA1-99B2-40A5-A4E9-9FBBAC380C60}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{407A8743-A532-48E3-9004-715BF423F4DA}">
   <ds:schemaRefs>

</xml_diff>